<commit_message>
Simplificar a 3 etapas y mostrar alimento por etapa en Inicio
Se reduce el esquema de etapas de 4 a 3 (Inicio: dias 1-21, Crecimiento:
dias 22-35, Engorde: dias 36-49), a peticion del usuario. Se agrega un
bloque en la hoja Inicio que muestra, apenas se ingresa la cantidad de
pollos, cuanto alimento (kg) y cuantos bultos comprar en cada una de las
tres etapas, sin tener que ir a otra hoja. Se aclara ademas en el rotulo
de "peso del bulto" que ese valor es el peso en kg de un bulto y no una
cantidad de bultos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LCh9wkrhUtgEqkX3z5Ds1d
</commit_message>
<xml_diff>
--- a/Control_Alimentacion_Pollos_Engorde.xlsx
+++ b/Control_Alimentacion_Pollos_Engorde.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="98">
   <si>
     <t xml:space="preserve">SISTEMA DE ALIMENTACIÓN AUTOMATIZADO — POLLOS DE ENGORDE</t>
   </si>
@@ -51,7 +51,7 @@
     <t xml:space="preserve">Peso del bulto de concentrado (kg):</t>
   </si>
   <si>
-    <t xml:space="preserve">Lista sugiere 40 o 50 kg; puede escribir otro peso</t>
+    <t xml:space="preserve">Es el peso en KG de 1 bulto (no la cantidad de bultos). La lista sugiere 40 o 50; puede escribir otro peso</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha de inicio del lote (día 1):</t>
@@ -66,7 +66,49 @@
     <t xml:space="preserve">Elija la semana que quiere ver en el resumen de abajo</t>
   </si>
   <si>
-    <t xml:space="preserve">2. RESULTADOS DE LA SEMANA SELECCIONADA</t>
+    <t xml:space="preserve">2. CUÁNTO ALIMENTO DAR POR ETAPA  (Inicio, Crecimiento, Engorde)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Etapa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Días</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alimento/ave
+etapa (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alimento total
+lote/etapa (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bultos a
+comprar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inicio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Días 1-21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crecimiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Días 22-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engorde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Días 36-49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL CICLO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. RESULTADOS DE LA SEMANA SELECCIONADA</t>
   </si>
   <si>
     <t xml:space="preserve">Etapa:</t>
@@ -99,7 +141,7 @@
     <t xml:space="preserve">Bultos acumulados hasta esa semana (redondeado):</t>
   </si>
   <si>
-    <t xml:space="preserve">3. RESUMEN DEL CICLO COMPLETO (SEMANA 1 A 7)</t>
+    <t xml:space="preserve">4. RESUMEN DEL CICLO COMPLETO (SEMANA 1 A 7)</t>
   </si>
   <si>
     <t xml:space="preserve">Consumo total por ave en todo el ciclo (kg):</t>
@@ -114,7 +156,7 @@
     <t xml:space="preserve">Total de bultos del ciclo — comprando semana a semana:</t>
   </si>
   <si>
-    <t xml:space="preserve">Consulte la hoja "Tabla Semanal" para ver el detalle de las 7 semanas y "Compra de Concentrado" para planificar la compra por etapa.</t>
+    <t xml:space="preserve">Consulte la hoja "Tabla Semanal" para ver el detalle de las 7 semanas y "Compra de Concentrado" para planificar la compra por etapa (incluye costos).</t>
   </si>
   <si>
     <t xml:space="preserve">TABLA SEMANAL DE CONSUMO — SEMANA 1 A 7</t>
@@ -124,9 +166,6 @@
   </si>
   <si>
     <t xml:space="preserve">Semana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Etapa</t>
   </si>
   <si>
     <t xml:space="preserve">Día
@@ -191,19 +230,7 @@
     <t xml:space="preserve">Fuente / Notas</t>
   </si>
   <si>
-    <t xml:space="preserve">Preiniciación</t>
-  </si>
-  <si>
     <t xml:space="preserve">Objetivos de desempeño típicos de líneas comerciales de engorde de alto rendimiento (Ross 308 / Cobb 500 — Aviagen / Cobb-Vantress), promediados a condiciones de campo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Iniciación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crecimiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Engorde</t>
   </si>
   <si>
     <t xml:space="preserve">IMPORTANTE: la columna "Consumo (g/ave/día)" es la única base numérica de todo el archivo. Todas las demás hojas (Tabla Semanal, Inicio, Registro Diario, Compra de Concentrado) calculan a partir de estos valores mediante fórmulas. Si su proveedor de concentrado (por ejemplo Italcol) le entrega una ficha técnica propia de consumo semanal para la línea genética que está manejando, reemplace aquí los valores de gramos/ave/día y el archivo se actualizará automáticamente.</t>
@@ -259,9 +286,6 @@
 incluidas</t>
   </si>
   <si>
-    <t xml:space="preserve">Días</t>
-  </si>
-  <si>
     <t xml:space="preserve">Consumo total
 etapa / ave (kg)</t>
   </si>
@@ -286,33 +310,15 @@
 etapa ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">Semana 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Días 1-7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Semanas 2-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Días 8-21</t>
+    <t xml:space="preserve">Semanas 1-3</t>
   </si>
   <si>
     <t xml:space="preserve">Semanas 4-5</t>
   </si>
   <si>
-    <t xml:space="preserve">Días 22-35</t>
-  </si>
-  <si>
     <t xml:space="preserve">Semanas 6-7</t>
   </si>
   <si>
-    <t xml:space="preserve">Días 36-49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL CICLO</t>
-  </si>
-  <si>
     <t xml:space="preserve">El precio por bulto (columna H) es opcional: si lo diligencia, el costo estimado se calcula solo. Si lo deja en 0, el costo total será 0.</t>
   </si>
   <si>
@@ -322,17 +328,17 @@
     <t xml:space="preserve">1. Cómo empezar</t>
   </si>
   <si>
-    <t xml:space="preserve">1) Vaya a la hoja "Inicio" y escriba la cantidad de pollos del lote (celda amarilla). 2) Verifique o cambie el peso del bulto (40, 50 u otro). 3) Escriba la fecha de inicio del lote. 4) Elija la semana que quiere consultar. Todos los cálculos del archivo se actualizan solos.</t>
+    <t xml:space="preserve">1) Vaya a la hoja "Inicio" y escriba la cantidad de pollos del lote (celda amarilla). 2) Verifique o cambie el peso del bulto (40, 50 u otro). 3) Escriba la fecha de inicio del lote. Justo debajo aparece cuánto alimento debe dar en cada etapa (Inicio, Crecimiento, Engorde). 4) Si además quiere el detalle semana a semana, elija la semana a consultar. Todo se actualiza solo.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Hojas del archivo</t>
   </si>
   <si>
-    <t xml:space="preserve">• Inicio: panel principal con los datos de entrada y el resumen de resultados.
+    <t xml:space="preserve">• Inicio: panel principal con los datos de entrada, cuánto alimento dar en cada etapa y el resumen de resultados.
 • Tabla Semanal: detalle completo de consumo, semana 1 a 7, con etapa, bultos y acumulados.
 • Tabla Tecnica Base: consumo de referencia en g/ave/día por semana (única hoja donde se edita el dato técnico base).
 • Registro Diario: para anotar el alimento suministrado y el sobrante cada día, y comparar contra lo calculado.
-• Compra de Concentrado: cuántos bultos comprar por cada etapa (preiniciación, iniciación, crecimiento, engorde).</t>
+• Compra de Concentrado: cuántos bultos comprar por cada etapa (Inicio, Crecimiento, Engorde), con costo estimado.</t>
   </si>
   <si>
     <t xml:space="preserve">3. Código de colores</t>
@@ -340,13 +346,13 @@
   <si>
     <t xml:space="preserve">• Celda amarilla con borde y letra azul: celda de ENTRADA. Aquí se escriben datos.
 • Celda blanca con letra negra: FÓRMULA. No se debe escribir sobre ella; se calcula sola.
-• Colores pastel (durazno, verde, azul, rosado): identifican visualmente cada etapa (preiniciación, iniciación, crecimiento, engorde).</t>
+• Colores pastel (durazno, azul, rosado): identifican visualmente cada etapa (Inicio, Crecimiento, Engorde).</t>
   </si>
   <si>
     <t xml:space="preserve">4. Nota técnica sobre la tabla de consumo</t>
   </si>
   <si>
-    <t xml:space="preserve">Los valores de gramos de alimento por ave/día (hoja "Tabla Tecnica Base") están basados en los objetivos de desempeño típicos publicados para las líneas comerciales de engorde de mayor uso a nivel mundial (Ross 308 de Aviagen y Cobb 500 de Cobb-Vantress), promediados y ajustados a condiciones comerciales de campo, ya que no se especificó una línea genética particular. Italcol, como la mayoría de las marcas de concentrado en Colombia, formula y recomienda sus programas de alimentación (preiniciador, iniciador, engorde/finalizador) sobre esta misma base técnica de las casas genéticas, por lo que esta tabla es una referencia válida para trabajar con concentrado Italcol. Si cuenta con la ficha técnica específica de Italcol para su programa (o con el dato exacto de la línea genética que está manejando), reemplácela en la columna E de la hoja "Tabla Tecnica Base": todo el archivo (Tabla Semanal, Inicio, Registro Diario y Compra de Concentrado) se recalculará automáticamente con los nuevos valores.</t>
+    <t xml:space="preserve">Los valores de gramos de alimento por ave/día (hoja "Tabla Tecnica Base") están basados en los objetivos de desempeño típicos publicados para las líneas comerciales de engorde de mayor uso a nivel mundial (Ross 308 de Aviagen y Cobb 500 de Cobb-Vantress), promediados y ajustados a condiciones comerciales de campo, ya que no se especificó una línea genética particular. Italcol, como la mayoría de las marcas de concentrado en Colombia, formula y recomienda sus programas de alimentación por etapas (inicio, crecimiento, engorde/finalizador) sobre esta misma base técnica de las casas genéticas, por lo que esta tabla es una referencia válida para trabajar con concentrado Italcol. Si cuenta con la ficha técnica específica de Italcol para su programa (o con el dato exacto de la línea genética que está manejando), reemplácela en la columna E de la hoja "Tabla Tecnica Base": todo el archivo (Tabla Semanal, Inicio, Registro Diario y Compra de Concentrado) se recalculará automáticamente con los nuevos valores.</t>
   </si>
   <si>
     <t xml:space="preserve">5. Supuestos del modelo</t>
@@ -433,13 +439,6 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -448,6 +447,13 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -485,7 +491,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -512,18 +518,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF2E3"/>
-        <bgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF375623"/>
         <bgColor rgb="FF1F5C2E"/>
       </patternFill>
@@ -532,12 +526,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFDEBD0"/>
         <bgColor rgb="FFFFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD5F5E3"/>
-        <bgColor rgb="FFD6EAF8"/>
       </patternFill>
     </fill>
     <fill>
@@ -556,6 +544,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1D3"/>
         <bgColor rgb="FFD6EAF8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF2E3"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -629,7 +629,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="64">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -662,23 +662,103 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -686,19 +766,55 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -706,103 +822,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -810,7 +846,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="13" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -826,39 +862,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="169" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="9" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1146,15 +1162,15 @@
     <tabColor rgb="FF1F5C2E"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1198,7 +1214,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
@@ -1241,160 +1257,266 @@
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="4" t="s">
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="8" t="str">
+      <c r="C11" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <f aca="false">'Compra de Concentrado'!D4</f>
+        <v>0.882</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <f aca="false">'Compra de Concentrado'!E4</f>
+        <v>88.2</v>
+      </c>
+      <c r="F12" s="13" t="n">
+        <f aca="false">'Compra de Concentrado'!G4</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <f aca="false">'Compra de Concentrado'!D5</f>
+        <v>1.47</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <f aca="false">'Compra de Concentrado'!E5</f>
+        <v>147</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <f aca="false">'Compra de Concentrado'!G5</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="21" t="n">
+        <f aca="false">'Compra de Concentrado'!D6</f>
+        <v>2.114</v>
+      </c>
+      <c r="E14" s="22" t="n">
+        <f aca="false">'Compra de Concentrado'!E6</f>
+        <v>211.4</v>
+      </c>
+      <c r="F14" s="23" t="n">
+        <f aca="false">'Compra de Concentrado'!G6</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="25"/>
+      <c r="D15" s="26" t="n">
+        <f aca="false">SUM(D12:D14)</f>
+        <v>4.466</v>
+      </c>
+      <c r="E15" s="26" t="n">
+        <f aca="false">SUM(E12:E14)</f>
+        <v>446.6</v>
+      </c>
+      <c r="F15" s="27" t="n">
+        <f aca="false">SUM(F12:F14)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="28" t="str">
         <f aca="false">INDEX('Tabla Semanal'!$B$4:$B$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))</f>
-        <v>Preiniciación</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="8" t="str">
+        <v>Inicio</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="28" t="str">
         <f aca="false">INDEX('Tabla Semanal'!$C$4:$C$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))&amp;" a "&amp;INDEX('Tabla Semanal'!$D$4:$D$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))&amp;" días"</f>
         <v>1 a 7 días</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" s="9" t="n">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="29" t="n">
         <f aca="false">INDEX('Tabla Semanal'!$E$4:$E$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))</f>
         <v>18</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="10" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="30" t="n">
         <f aca="false">INDEX('Tabla Semanal'!$F$4:$F$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))</f>
         <v>0.018</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="11" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="31" t="n">
         <f aca="false">INDEX('Tabla Semanal'!$G$4:$G$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))</f>
         <v>1.8</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="11" t="n">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="31" t="n">
         <f aca="false">INDEX('Tabla Semanal'!$H$4:$H$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))</f>
         <v>12.6</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="10" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D24" s="30" t="n">
         <f aca="false">INDEX('Tabla Semanal'!$I$4:$I$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))</f>
         <v>0.315</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="12" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="32" t="n">
         <f aca="false">INDEX('Tabla Semanal'!$J$4:$J$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" s="11" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="31" t="n">
         <f aca="false">INDEX('Tabla Semanal'!$K$4:$K$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))</f>
         <v>12.6</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D20" s="9" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D27" s="29" t="n">
         <f aca="false">INDEX('Tabla Semanal'!$M$4:$M$10,MATCH(SemanaConsulta,'Tabla Semanal'!$A$4:$A$10,0))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D23" s="11" t="n">
-        <f aca="false">D24/CantidadPollos</f>
+    <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D30" s="31" t="n">
+        <f aca="false">D31/CantidadPollos</f>
         <v>4.466</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D24" s="11" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D31" s="31" t="n">
         <f aca="false">'Tabla Semanal'!$K$10</f>
         <v>446.6</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25" s="12" t="n">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D32" s="32" t="n">
         <f aca="false">'Tabla Semanal'!$M$10</f>
         <v>12</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D26" s="12" t="n">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D33" s="32" t="n">
         <f aca="false">'Tabla Semanal'!$J$11</f>
         <v>15</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="33"/>
+      <c r="E35" s="33"/>
+      <c r="F35" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A35:F35"/>
   </mergeCells>
   <dataValidations count="3">
     <dataValidation allowBlank="false" error="Lo habitual es 40 o 50 kg. Puede continuar con otro valor si su presentación es diferente." errorStyle="warning" errorTitle="Peso de bulto inusual" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D6" type="list">
@@ -1443,25 +1565,25 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
+      <c r="A1" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1477,441 +1599,441 @@
       <c r="M2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="J3" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="L3" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="M3" s="15" t="s">
-        <v>42</v>
+      <c r="A3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="n">
+      <c r="A4" s="35" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="17" t="str">
+      <c r="B4" s="36" t="str">
         <f aca="false">INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(A4,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
-        <v>Preiniciación</v>
-      </c>
-      <c r="C4" s="18" t="n">
+        <v>Inicio</v>
+      </c>
+      <c r="C4" s="37" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$C$4:$C$10,MATCH(A4,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>1</v>
       </c>
-      <c r="D4" s="18" t="n">
+      <c r="D4" s="37" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$D$4:$D$10,MATCH(A4,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>7</v>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="37" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(A4,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>18</v>
       </c>
-      <c r="F4" s="19" t="n">
+      <c r="F4" s="38" t="n">
         <f aca="false">E4/1000</f>
         <v>0.018</v>
       </c>
-      <c r="G4" s="19" t="n">
+      <c r="G4" s="38" t="n">
         <f aca="false">F4*CantidadPollos</f>
         <v>1.8</v>
       </c>
-      <c r="H4" s="20" t="n">
+      <c r="H4" s="39" t="n">
         <f aca="false">G4*7</f>
         <v>12.6</v>
       </c>
-      <c r="I4" s="19" t="n">
+      <c r="I4" s="38" t="n">
         <f aca="false">H4/PesoBulto</f>
         <v>0.315</v>
       </c>
-      <c r="J4" s="21" t="n">
+      <c r="J4" s="40" t="n">
         <f aca="false">ROUNDUP(I4,0)</f>
         <v>1</v>
       </c>
-      <c r="K4" s="20" t="n">
+      <c r="K4" s="39" t="n">
         <f aca="false">H4</f>
         <v>12.6</v>
       </c>
-      <c r="L4" s="19" t="n">
+      <c r="L4" s="38" t="n">
         <f aca="false">K4/PesoBulto</f>
         <v>0.315</v>
       </c>
-      <c r="M4" s="22" t="n">
+      <c r="M4" s="41" t="n">
         <f aca="false">ROUNDUP(L4,0)</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="n">
+      <c r="A5" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="24" t="str">
+      <c r="B5" s="36" t="str">
         <f aca="false">INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(A5,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
-        <v>Iniciación</v>
-      </c>
-      <c r="C5" s="25" t="n">
+        <v>Inicio</v>
+      </c>
+      <c r="C5" s="37" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$C$4:$C$10,MATCH(A5,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>8</v>
       </c>
-      <c r="D5" s="25" t="n">
+      <c r="D5" s="37" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$D$4:$D$10,MATCH(A5,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>14</v>
       </c>
-      <c r="E5" s="25" t="n">
+      <c r="E5" s="37" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(A5,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>42</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="38" t="n">
         <f aca="false">E5/1000</f>
         <v>0.042</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="38" t="n">
         <f aca="false">F5*CantidadPollos</f>
         <v>4.2</v>
       </c>
-      <c r="H5" s="20" t="n">
+      <c r="H5" s="39" t="n">
         <f aca="false">G5*7</f>
         <v>29.4</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="38" t="n">
         <f aca="false">H5/PesoBulto</f>
         <v>0.735</v>
       </c>
-      <c r="J5" s="21" t="n">
+      <c r="J5" s="40" t="n">
         <f aca="false">ROUNDUP(I5,0)</f>
         <v>1</v>
       </c>
-      <c r="K5" s="20" t="n">
+      <c r="K5" s="39" t="n">
         <f aca="false">K4+H5</f>
         <v>42</v>
       </c>
-      <c r="L5" s="19" t="n">
+      <c r="L5" s="38" t="n">
         <f aca="false">K5/PesoBulto</f>
         <v>1.05</v>
       </c>
-      <c r="M5" s="22" t="n">
+      <c r="M5" s="41" t="n">
         <f aca="false">ROUNDUP(L5,0)</f>
         <v>2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="n">
+      <c r="A6" s="35" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="24" t="str">
+      <c r="B6" s="36" t="str">
         <f aca="false">INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(A6,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
-        <v>Iniciación</v>
-      </c>
-      <c r="C6" s="25" t="n">
+        <v>Inicio</v>
+      </c>
+      <c r="C6" s="37" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$C$4:$C$10,MATCH(A6,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>15</v>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D6" s="37" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$D$4:$D$10,MATCH(A6,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>21</v>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E6" s="37" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(A6,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>66</v>
       </c>
-      <c r="F6" s="19" t="n">
+      <c r="F6" s="38" t="n">
         <f aca="false">E6/1000</f>
         <v>0.066</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G6" s="38" t="n">
         <f aca="false">F6*CantidadPollos</f>
         <v>6.6</v>
       </c>
-      <c r="H6" s="20" t="n">
+      <c r="H6" s="39" t="n">
         <f aca="false">G6*7</f>
         <v>46.2</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I6" s="38" t="n">
         <f aca="false">H6/PesoBulto</f>
         <v>1.155</v>
       </c>
-      <c r="J6" s="21" t="n">
+      <c r="J6" s="40" t="n">
         <f aca="false">ROUNDUP(I6,0)</f>
         <v>2</v>
       </c>
-      <c r="K6" s="20" t="n">
+      <c r="K6" s="39" t="n">
         <f aca="false">K5+H6</f>
         <v>88.2</v>
       </c>
-      <c r="L6" s="19" t="n">
+      <c r="L6" s="38" t="n">
         <f aca="false">K6/PesoBulto</f>
         <v>2.205</v>
       </c>
-      <c r="M6" s="22" t="n">
+      <c r="M6" s="41" t="n">
         <f aca="false">ROUNDUP(L6,0)</f>
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="26" t="n">
+      <c r="A7" s="42" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="27" t="str">
+      <c r="B7" s="43" t="str">
         <f aca="false">INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(A7,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>Crecimiento</v>
       </c>
-      <c r="C7" s="28" t="n">
+      <c r="C7" s="44" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$C$4:$C$10,MATCH(A7,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>22</v>
       </c>
-      <c r="D7" s="28" t="n">
+      <c r="D7" s="44" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$D$4:$D$10,MATCH(A7,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>28</v>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E7" s="44" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(A7,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>92</v>
       </c>
-      <c r="F7" s="19" t="n">
+      <c r="F7" s="38" t="n">
         <f aca="false">E7/1000</f>
         <v>0.092</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="38" t="n">
         <f aca="false">F7*CantidadPollos</f>
         <v>9.2</v>
       </c>
-      <c r="H7" s="20" t="n">
+      <c r="H7" s="39" t="n">
         <f aca="false">G7*7</f>
         <v>64.4</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="38" t="n">
         <f aca="false">H7/PesoBulto</f>
         <v>1.61</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="J7" s="40" t="n">
         <f aca="false">ROUNDUP(I7,0)</f>
         <v>2</v>
       </c>
-      <c r="K7" s="20" t="n">
+      <c r="K7" s="39" t="n">
         <f aca="false">K6+H7</f>
         <v>152.6</v>
       </c>
-      <c r="L7" s="19" t="n">
+      <c r="L7" s="38" t="n">
         <f aca="false">K7/PesoBulto</f>
         <v>3.815</v>
       </c>
-      <c r="M7" s="22" t="n">
+      <c r="M7" s="41" t="n">
         <f aca="false">ROUNDUP(L7,0)</f>
         <v>4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="n">
+      <c r="A8" s="42" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="27" t="str">
+      <c r="B8" s="43" t="str">
         <f aca="false">INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(A8,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>Crecimiento</v>
       </c>
-      <c r="C8" s="28" t="n">
+      <c r="C8" s="44" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$C$4:$C$10,MATCH(A8,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>29</v>
       </c>
-      <c r="D8" s="28" t="n">
+      <c r="D8" s="44" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$D$4:$D$10,MATCH(A8,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>35</v>
       </c>
-      <c r="E8" s="28" t="n">
+      <c r="E8" s="44" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(A8,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>118</v>
       </c>
-      <c r="F8" s="19" t="n">
+      <c r="F8" s="38" t="n">
         <f aca="false">E8/1000</f>
         <v>0.118</v>
       </c>
-      <c r="G8" s="19" t="n">
+      <c r="G8" s="38" t="n">
         <f aca="false">F8*CantidadPollos</f>
         <v>11.8</v>
       </c>
-      <c r="H8" s="20" t="n">
+      <c r="H8" s="39" t="n">
         <f aca="false">G8*7</f>
         <v>82.6</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="38" t="n">
         <f aca="false">H8/PesoBulto</f>
         <v>2.065</v>
       </c>
-      <c r="J8" s="21" t="n">
+      <c r="J8" s="40" t="n">
         <f aca="false">ROUNDUP(I8,0)</f>
         <v>3</v>
       </c>
-      <c r="K8" s="20" t="n">
+      <c r="K8" s="39" t="n">
         <f aca="false">K7+H8</f>
         <v>235.2</v>
       </c>
-      <c r="L8" s="19" t="n">
+      <c r="L8" s="38" t="n">
         <f aca="false">K8/PesoBulto</f>
         <v>5.88</v>
       </c>
-      <c r="M8" s="22" t="n">
+      <c r="M8" s="41" t="n">
         <f aca="false">ROUNDUP(L8,0)</f>
         <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="29" t="n">
+      <c r="A9" s="45" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="30" t="str">
+      <c r="B9" s="46" t="str">
         <f aca="false">INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(A9,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>Engorde</v>
       </c>
-      <c r="C9" s="31" t="n">
+      <c r="C9" s="47" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$C$4:$C$10,MATCH(A9,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>36</v>
       </c>
-      <c r="D9" s="31" t="n">
+      <c r="D9" s="47" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$D$4:$D$10,MATCH(A9,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>42</v>
       </c>
-      <c r="E9" s="31" t="n">
+      <c r="E9" s="47" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(A9,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>142</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="38" t="n">
         <f aca="false">E9/1000</f>
         <v>0.142</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="38" t="n">
         <f aca="false">F9*CantidadPollos</f>
         <v>14.2</v>
       </c>
-      <c r="H9" s="20" t="n">
+      <c r="H9" s="39" t="n">
         <f aca="false">G9*7</f>
         <v>99.4</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="I9" s="38" t="n">
         <f aca="false">H9/PesoBulto</f>
         <v>2.485</v>
       </c>
-      <c r="J9" s="21" t="n">
+      <c r="J9" s="40" t="n">
         <f aca="false">ROUNDUP(I9,0)</f>
         <v>3</v>
       </c>
-      <c r="K9" s="20" t="n">
+      <c r="K9" s="39" t="n">
         <f aca="false">K8+H9</f>
         <v>334.6</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="L9" s="38" t="n">
         <f aca="false">K9/PesoBulto</f>
         <v>8.365</v>
       </c>
-      <c r="M9" s="22" t="n">
+      <c r="M9" s="41" t="n">
         <f aca="false">ROUNDUP(L9,0)</f>
         <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="29" t="n">
+      <c r="A10" s="45" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="30" t="str">
+      <c r="B10" s="46" t="str">
         <f aca="false">INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(A10,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>Engorde</v>
       </c>
-      <c r="C10" s="31" t="n">
+      <c r="C10" s="47" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$C$4:$C$10,MATCH(A10,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>43</v>
       </c>
-      <c r="D10" s="31" t="n">
+      <c r="D10" s="47" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$D$4:$D$10,MATCH(A10,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>49</v>
       </c>
-      <c r="E10" s="31" t="n">
+      <c r="E10" s="47" t="n">
         <f aca="false">INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(A10,'Tabla Tecnica Base'!$A$4:$A$10,0))</f>
         <v>160</v>
       </c>
-      <c r="F10" s="19" t="n">
+      <c r="F10" s="38" t="n">
         <f aca="false">E10/1000</f>
         <v>0.16</v>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="38" t="n">
         <f aca="false">F10*CantidadPollos</f>
         <v>16</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="39" t="n">
         <f aca="false">G10*7</f>
         <v>112</v>
       </c>
-      <c r="I10" s="19" t="n">
+      <c r="I10" s="38" t="n">
         <f aca="false">H10/PesoBulto</f>
         <v>2.8</v>
       </c>
-      <c r="J10" s="21" t="n">
+      <c r="J10" s="40" t="n">
         <f aca="false">ROUNDUP(I10,0)</f>
         <v>3</v>
       </c>
-      <c r="K10" s="20" t="n">
+      <c r="K10" s="39" t="n">
         <f aca="false">K9+H10</f>
         <v>446.6</v>
       </c>
-      <c r="L10" s="19" t="n">
+      <c r="L10" s="38" t="n">
         <f aca="false">K10/PesoBulto</f>
         <v>11.165</v>
       </c>
-      <c r="M10" s="22" t="n">
+      <c r="M10" s="41" t="n">
         <f aca="false">ROUNDUP(L10,0)</f>
         <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="33"/>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="33"/>
-      <c r="H11" s="34" t="n">
+      <c r="A11" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="25"/>
+      <c r="C11" s="25"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="25"/>
+      <c r="H11" s="26" t="n">
         <f aca="false">SUM(H4:H10)</f>
         <v>446.6</v>
       </c>
-      <c r="I11" s="35"/>
-      <c r="J11" s="36" t="n">
+      <c r="I11" s="49"/>
+      <c r="J11" s="27" t="n">
         <f aca="false">SUM(J4:J10)</f>
         <v>15</v>
       </c>
-      <c r="K11" s="34" t="n">
+      <c r="K11" s="26" t="n">
         <f aca="false">K10</f>
         <v>446.6</v>
       </c>
-      <c r="L11" s="35"/>
-      <c r="M11" s="36" t="n">
+      <c r="L11" s="49"/>
+      <c r="M11" s="27" t="n">
         <f aca="false">M10</f>
         <v>12</v>
       </c>
@@ -1949,18 +2071,18 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
+      <c r="A1" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1969,198 +2091,198 @@
       <c r="F2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="15" t="s">
+      <c r="A3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>48</v>
+      <c r="F3" s="8" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="37" t="n">
+      <c r="A4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="C4" s="37" t="n">
+      <c r="B4" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="37" t="n">
+      <c r="D4" s="10" t="n">
         <v>7</v>
       </c>
       <c r="E4" s="5" t="n">
         <v>18</v>
       </c>
-      <c r="F4" s="38" t="s">
-        <v>50</v>
+      <c r="F4" s="50" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="39" t="n">
+      <c r="A5" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="C5" s="39" t="n">
+      <c r="B5" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="D5" s="39" t="n">
+      <c r="D5" s="10" t="n">
         <v>14</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="F5" s="38" t="s">
-        <v>50</v>
+      <c r="F5" s="50" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="39" t="n">
+      <c r="A6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="39" t="n">
+      <c r="B6" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="D6" s="39" t="n">
+      <c r="D6" s="10" t="n">
         <v>21</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>66</v>
       </c>
-      <c r="F6" s="38" t="s">
-        <v>50</v>
+      <c r="F6" s="50" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="40" t="n">
+      <c r="A7" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" s="40" t="n">
+      <c r="B7" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="15" t="n">
         <v>22</v>
       </c>
-      <c r="D7" s="40" t="n">
+      <c r="D7" s="15" t="n">
         <v>28</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>92</v>
       </c>
-      <c r="F7" s="38" t="s">
-        <v>50</v>
+      <c r="F7" s="50" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="40" t="n">
+      <c r="A8" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="40" t="n">
+      <c r="B8" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="15" t="n">
         <v>29</v>
       </c>
-      <c r="D8" s="40" t="n">
+      <c r="D8" s="15" t="n">
         <v>35</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>118</v>
       </c>
-      <c r="F8" s="38" t="s">
-        <v>50</v>
+      <c r="F8" s="50" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="41" t="n">
+      <c r="A9" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="41" t="n">
+      <c r="B9" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="D9" s="41" t="n">
+      <c r="D9" s="20" t="n">
         <v>42</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>142</v>
       </c>
-      <c r="F9" s="38" t="s">
-        <v>50</v>
+      <c r="F9" s="50" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="41" t="n">
+      <c r="A10" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="41" t="n">
+      <c r="B10" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="20" t="n">
         <v>43</v>
       </c>
-      <c r="D10" s="41" t="n">
+      <c r="D10" s="20" t="n">
         <v>49</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>160</v>
       </c>
-      <c r="F10" s="38" t="s">
-        <v>50</v>
+      <c r="F10" s="50" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="42" t="s">
-        <v>54</v>
-      </c>
-      <c r="B12" s="42"/>
-      <c r="C12" s="42"/>
-      <c r="D12" s="42"/>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
+      <c r="A12" s="51" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="51"/>
+      <c r="C12" s="51"/>
+      <c r="D12" s="51"/>
+      <c r="E12" s="51"/>
+      <c r="F12" s="51"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="42"/>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="42"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
+      <c r="A13" s="51"/>
+      <c r="B13" s="51"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="51"/>
+      <c r="E13" s="51"/>
+      <c r="F13" s="51"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="42"/>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="42"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="42"/>
+      <c r="A14" s="51"/>
+      <c r="B14" s="51"/>
+      <c r="C14" s="51"/>
+      <c r="D14" s="51"/>
+      <c r="E14" s="51"/>
+      <c r="F14" s="51"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="42"/>
-      <c r="B15" s="42"/>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
+      <c r="A15" s="51"/>
+      <c r="B15" s="51"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="51"/>
+      <c r="F15" s="51"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2199,22 +2321,22 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
+      <c r="A1" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2227,1857 +2349,1857 @@
       <c r="J2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="H4" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="J4" s="15" t="s">
-        <v>64</v>
+      <c r="A4" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="43" t="n">
+      <c r="A5" s="52" t="n">
         <v>46285</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="41" t="n">
         <f aca="false">IF(A5="","",A5-FechaInicioLote+1)</f>
         <v>1</v>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="41" t="n">
         <f aca="false">IF(A5="","",MIN(7,MAX(1,ROUNDUP(B5/7,0))))</f>
         <v>1</v>
       </c>
-      <c r="D5" s="44" t="str">
+      <c r="D5" s="53" t="str">
         <f aca="false">IF(A5="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C5,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
-        <v>Preiniciación</v>
-      </c>
-      <c r="E5" s="45" t="n">
+        <v>Inicio</v>
+      </c>
+      <c r="E5" s="54" t="n">
         <v>2.5</v>
       </c>
-      <c r="F5" s="45" t="n">
+      <c r="F5" s="54" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="38" t="n">
         <f aca="false">IF(E5="","",E5-IF(F5="",0,F5))</f>
         <v>2.3</v>
       </c>
-      <c r="H5" s="19" t="n">
+      <c r="H5" s="38" t="n">
         <f aca="false">IF(A5="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C5,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v>1.8</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="38" t="n">
         <f aca="false">IF(OR(G5="",H5=""),"",G5-H5)</f>
         <v>0.5</v>
       </c>
-      <c r="J5" s="46" t="n">
+      <c r="J5" s="55" t="n">
         <f aca="false">IF(OR(I5="",H5="",H5=0),"",I5/H5)</f>
         <v>0.277777777777778</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="47"/>
-      <c r="B6" s="22" t="str">
+      <c r="A6" s="56"/>
+      <c r="B6" s="41" t="str">
         <f aca="false">IF(A6="","",A6-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C6" s="22" t="str">
+      <c r="C6" s="41" t="str">
         <f aca="false">IF(A6="","",MIN(7,MAX(1,ROUNDUP(B6/7,0))))</f>
         <v/>
       </c>
-      <c r="D6" s="44" t="str">
+      <c r="D6" s="53" t="str">
         <f aca="false">IF(A6="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C6,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E6" s="48"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="19" t="str">
+      <c r="E6" s="57"/>
+      <c r="F6" s="57"/>
+      <c r="G6" s="38" t="str">
         <f aca="false">IF(E6="","",E6-IF(F6="",0,F6))</f>
         <v/>
       </c>
-      <c r="H6" s="19" t="str">
+      <c r="H6" s="38" t="str">
         <f aca="false">IF(A6="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C6,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I6" s="19" t="str">
+      <c r="I6" s="38" t="str">
         <f aca="false">IF(OR(G6="",H6=""),"",G6-H6)</f>
         <v/>
       </c>
-      <c r="J6" s="46" t="str">
+      <c r="J6" s="55" t="str">
         <f aca="false">IF(OR(I6="",H6="",H6=0),"",I6/H6)</f>
         <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="47"/>
-      <c r="B7" s="22" t="str">
+      <c r="A7" s="56"/>
+      <c r="B7" s="41" t="str">
         <f aca="false">IF(A7="","",A7-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C7" s="22" t="str">
+      <c r="C7" s="41" t="str">
         <f aca="false">IF(A7="","",MIN(7,MAX(1,ROUNDUP(B7/7,0))))</f>
         <v/>
       </c>
-      <c r="D7" s="44" t="str">
+      <c r="D7" s="53" t="str">
         <f aca="false">IF(A7="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C7,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E7" s="48"/>
-      <c r="F7" s="48"/>
-      <c r="G7" s="19" t="str">
+      <c r="E7" s="57"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="38" t="str">
         <f aca="false">IF(E7="","",E7-IF(F7="",0,F7))</f>
         <v/>
       </c>
-      <c r="H7" s="19" t="str">
+      <c r="H7" s="38" t="str">
         <f aca="false">IF(A7="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C7,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I7" s="19" t="str">
+      <c r="I7" s="38" t="str">
         <f aca="false">IF(OR(G7="",H7=""),"",G7-H7)</f>
         <v/>
       </c>
-      <c r="J7" s="46" t="str">
+      <c r="J7" s="55" t="str">
         <f aca="false">IF(OR(I7="",H7="",H7=0),"",I7/H7)</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="47"/>
-      <c r="B8" s="22" t="str">
+      <c r="A8" s="56"/>
+      <c r="B8" s="41" t="str">
         <f aca="false">IF(A8="","",A8-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C8" s="22" t="str">
+      <c r="C8" s="41" t="str">
         <f aca="false">IF(A8="","",MIN(7,MAX(1,ROUNDUP(B8/7,0))))</f>
         <v/>
       </c>
-      <c r="D8" s="44" t="str">
+      <c r="D8" s="53" t="str">
         <f aca="false">IF(A8="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C8,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="19" t="str">
+      <c r="E8" s="57"/>
+      <c r="F8" s="57"/>
+      <c r="G8" s="38" t="str">
         <f aca="false">IF(E8="","",E8-IF(F8="",0,F8))</f>
         <v/>
       </c>
-      <c r="H8" s="19" t="str">
+      <c r="H8" s="38" t="str">
         <f aca="false">IF(A8="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C8,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I8" s="19" t="str">
+      <c r="I8" s="38" t="str">
         <f aca="false">IF(OR(G8="",H8=""),"",G8-H8)</f>
         <v/>
       </c>
-      <c r="J8" s="46" t="str">
+      <c r="J8" s="55" t="str">
         <f aca="false">IF(OR(I8="",H8="",H8=0),"",I8/H8)</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="47"/>
-      <c r="B9" s="22" t="str">
+      <c r="A9" s="56"/>
+      <c r="B9" s="41" t="str">
         <f aca="false">IF(A9="","",A9-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C9" s="22" t="str">
+      <c r="C9" s="41" t="str">
         <f aca="false">IF(A9="","",MIN(7,MAX(1,ROUNDUP(B9/7,0))))</f>
         <v/>
       </c>
-      <c r="D9" s="44" t="str">
+      <c r="D9" s="53" t="str">
         <f aca="false">IF(A9="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C9,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E9" s="48"/>
-      <c r="F9" s="48"/>
-      <c r="G9" s="19" t="str">
+      <c r="E9" s="57"/>
+      <c r="F9" s="57"/>
+      <c r="G9" s="38" t="str">
         <f aca="false">IF(E9="","",E9-IF(F9="",0,F9))</f>
         <v/>
       </c>
-      <c r="H9" s="19" t="str">
+      <c r="H9" s="38" t="str">
         <f aca="false">IF(A9="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C9,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I9" s="19" t="str">
+      <c r="I9" s="38" t="str">
         <f aca="false">IF(OR(G9="",H9=""),"",G9-H9)</f>
         <v/>
       </c>
-      <c r="J9" s="46" t="str">
+      <c r="J9" s="55" t="str">
         <f aca="false">IF(OR(I9="",H9="",H9=0),"",I9/H9)</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="47"/>
-      <c r="B10" s="22" t="str">
+      <c r="A10" s="56"/>
+      <c r="B10" s="41" t="str">
         <f aca="false">IF(A10="","",A10-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C10" s="22" t="str">
+      <c r="C10" s="41" t="str">
         <f aca="false">IF(A10="","",MIN(7,MAX(1,ROUNDUP(B10/7,0))))</f>
         <v/>
       </c>
-      <c r="D10" s="44" t="str">
+      <c r="D10" s="53" t="str">
         <f aca="false">IF(A10="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C10,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
-      <c r="G10" s="19" t="str">
+      <c r="E10" s="57"/>
+      <c r="F10" s="57"/>
+      <c r="G10" s="38" t="str">
         <f aca="false">IF(E10="","",E10-IF(F10="",0,F10))</f>
         <v/>
       </c>
-      <c r="H10" s="19" t="str">
+      <c r="H10" s="38" t="str">
         <f aca="false">IF(A10="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C10,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I10" s="19" t="str">
+      <c r="I10" s="38" t="str">
         <f aca="false">IF(OR(G10="",H10=""),"",G10-H10)</f>
         <v/>
       </c>
-      <c r="J10" s="46" t="str">
+      <c r="J10" s="55" t="str">
         <f aca="false">IF(OR(I10="",H10="",H10=0),"",I10/H10)</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="47"/>
-      <c r="B11" s="22" t="str">
+      <c r="A11" s="56"/>
+      <c r="B11" s="41" t="str">
         <f aca="false">IF(A11="","",A11-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C11" s="22" t="str">
+      <c r="C11" s="41" t="str">
         <f aca="false">IF(A11="","",MIN(7,MAX(1,ROUNDUP(B11/7,0))))</f>
         <v/>
       </c>
-      <c r="D11" s="44" t="str">
+      <c r="D11" s="53" t="str">
         <f aca="false">IF(A11="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C11,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E11" s="48"/>
-      <c r="F11" s="48"/>
-      <c r="G11" s="19" t="str">
+      <c r="E11" s="57"/>
+      <c r="F11" s="57"/>
+      <c r="G11" s="38" t="str">
         <f aca="false">IF(E11="","",E11-IF(F11="",0,F11))</f>
         <v/>
       </c>
-      <c r="H11" s="19" t="str">
+      <c r="H11" s="38" t="str">
         <f aca="false">IF(A11="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C11,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I11" s="19" t="str">
+      <c r="I11" s="38" t="str">
         <f aca="false">IF(OR(G11="",H11=""),"",G11-H11)</f>
         <v/>
       </c>
-      <c r="J11" s="46" t="str">
+      <c r="J11" s="55" t="str">
         <f aca="false">IF(OR(I11="",H11="",H11=0),"",I11/H11)</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="47"/>
-      <c r="B12" s="22" t="str">
+      <c r="A12" s="56"/>
+      <c r="B12" s="41" t="str">
         <f aca="false">IF(A12="","",A12-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C12" s="22" t="str">
+      <c r="C12" s="41" t="str">
         <f aca="false">IF(A12="","",MIN(7,MAX(1,ROUNDUP(B12/7,0))))</f>
         <v/>
       </c>
-      <c r="D12" s="44" t="str">
+      <c r="D12" s="53" t="str">
         <f aca="false">IF(A12="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C12,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E12" s="48"/>
-      <c r="F12" s="48"/>
-      <c r="G12" s="19" t="str">
+      <c r="E12" s="57"/>
+      <c r="F12" s="57"/>
+      <c r="G12" s="38" t="str">
         <f aca="false">IF(E12="","",E12-IF(F12="",0,F12))</f>
         <v/>
       </c>
-      <c r="H12" s="19" t="str">
+      <c r="H12" s="38" t="str">
         <f aca="false">IF(A12="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C12,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I12" s="19" t="str">
+      <c r="I12" s="38" t="str">
         <f aca="false">IF(OR(G12="",H12=""),"",G12-H12)</f>
         <v/>
       </c>
-      <c r="J12" s="46" t="str">
+      <c r="J12" s="55" t="str">
         <f aca="false">IF(OR(I12="",H12="",H12=0),"",I12/H12)</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="47"/>
-      <c r="B13" s="22" t="str">
+      <c r="A13" s="56"/>
+      <c r="B13" s="41" t="str">
         <f aca="false">IF(A13="","",A13-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C13" s="22" t="str">
+      <c r="C13" s="41" t="str">
         <f aca="false">IF(A13="","",MIN(7,MAX(1,ROUNDUP(B13/7,0))))</f>
         <v/>
       </c>
-      <c r="D13" s="44" t="str">
+      <c r="D13" s="53" t="str">
         <f aca="false">IF(A13="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C13,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E13" s="48"/>
-      <c r="F13" s="48"/>
-      <c r="G13" s="19" t="str">
+      <c r="E13" s="57"/>
+      <c r="F13" s="57"/>
+      <c r="G13" s="38" t="str">
         <f aca="false">IF(E13="","",E13-IF(F13="",0,F13))</f>
         <v/>
       </c>
-      <c r="H13" s="19" t="str">
+      <c r="H13" s="38" t="str">
         <f aca="false">IF(A13="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C13,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I13" s="19" t="str">
+      <c r="I13" s="38" t="str">
         <f aca="false">IF(OR(G13="",H13=""),"",G13-H13)</f>
         <v/>
       </c>
-      <c r="J13" s="46" t="str">
+      <c r="J13" s="55" t="str">
         <f aca="false">IF(OR(I13="",H13="",H13=0),"",I13/H13)</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="47"/>
-      <c r="B14" s="22" t="str">
+      <c r="A14" s="56"/>
+      <c r="B14" s="41" t="str">
         <f aca="false">IF(A14="","",A14-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C14" s="22" t="str">
+      <c r="C14" s="41" t="str">
         <f aca="false">IF(A14="","",MIN(7,MAX(1,ROUNDUP(B14/7,0))))</f>
         <v/>
       </c>
-      <c r="D14" s="44" t="str">
+      <c r="D14" s="53" t="str">
         <f aca="false">IF(A14="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C14,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E14" s="48"/>
-      <c r="F14" s="48"/>
-      <c r="G14" s="19" t="str">
+      <c r="E14" s="57"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="38" t="str">
         <f aca="false">IF(E14="","",E14-IF(F14="",0,F14))</f>
         <v/>
       </c>
-      <c r="H14" s="19" t="str">
+      <c r="H14" s="38" t="str">
         <f aca="false">IF(A14="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C14,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I14" s="19" t="str">
+      <c r="I14" s="38" t="str">
         <f aca="false">IF(OR(G14="",H14=""),"",G14-H14)</f>
         <v/>
       </c>
-      <c r="J14" s="46" t="str">
+      <c r="J14" s="55" t="str">
         <f aca="false">IF(OR(I14="",H14="",H14=0),"",I14/H14)</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="47"/>
-      <c r="B15" s="22" t="str">
+      <c r="A15" s="56"/>
+      <c r="B15" s="41" t="str">
         <f aca="false">IF(A15="","",A15-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C15" s="22" t="str">
+      <c r="C15" s="41" t="str">
         <f aca="false">IF(A15="","",MIN(7,MAX(1,ROUNDUP(B15/7,0))))</f>
         <v/>
       </c>
-      <c r="D15" s="44" t="str">
+      <c r="D15" s="53" t="str">
         <f aca="false">IF(A15="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C15,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E15" s="48"/>
-      <c r="F15" s="48"/>
-      <c r="G15" s="19" t="str">
+      <c r="E15" s="57"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="38" t="str">
         <f aca="false">IF(E15="","",E15-IF(F15="",0,F15))</f>
         <v/>
       </c>
-      <c r="H15" s="19" t="str">
+      <c r="H15" s="38" t="str">
         <f aca="false">IF(A15="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C15,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I15" s="19" t="str">
+      <c r="I15" s="38" t="str">
         <f aca="false">IF(OR(G15="",H15=""),"",G15-H15)</f>
         <v/>
       </c>
-      <c r="J15" s="46" t="str">
+      <c r="J15" s="55" t="str">
         <f aca="false">IF(OR(I15="",H15="",H15=0),"",I15/H15)</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="47"/>
-      <c r="B16" s="22" t="str">
+      <c r="A16" s="56"/>
+      <c r="B16" s="41" t="str">
         <f aca="false">IF(A16="","",A16-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C16" s="22" t="str">
+      <c r="C16" s="41" t="str">
         <f aca="false">IF(A16="","",MIN(7,MAX(1,ROUNDUP(B16/7,0))))</f>
         <v/>
       </c>
-      <c r="D16" s="44" t="str">
+      <c r="D16" s="53" t="str">
         <f aca="false">IF(A16="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C16,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E16" s="48"/>
-      <c r="F16" s="48"/>
-      <c r="G16" s="19" t="str">
+      <c r="E16" s="57"/>
+      <c r="F16" s="57"/>
+      <c r="G16" s="38" t="str">
         <f aca="false">IF(E16="","",E16-IF(F16="",0,F16))</f>
         <v/>
       </c>
-      <c r="H16" s="19" t="str">
+      <c r="H16" s="38" t="str">
         <f aca="false">IF(A16="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C16,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I16" s="19" t="str">
+      <c r="I16" s="38" t="str">
         <f aca="false">IF(OR(G16="",H16=""),"",G16-H16)</f>
         <v/>
       </c>
-      <c r="J16" s="46" t="str">
+      <c r="J16" s="55" t="str">
         <f aca="false">IF(OR(I16="",H16="",H16=0),"",I16/H16)</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="47"/>
-      <c r="B17" s="22" t="str">
+      <c r="A17" s="56"/>
+      <c r="B17" s="41" t="str">
         <f aca="false">IF(A17="","",A17-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C17" s="22" t="str">
+      <c r="C17" s="41" t="str">
         <f aca="false">IF(A17="","",MIN(7,MAX(1,ROUNDUP(B17/7,0))))</f>
         <v/>
       </c>
-      <c r="D17" s="44" t="str">
+      <c r="D17" s="53" t="str">
         <f aca="false">IF(A17="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C17,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E17" s="48"/>
-      <c r="F17" s="48"/>
-      <c r="G17" s="19" t="str">
+      <c r="E17" s="57"/>
+      <c r="F17" s="57"/>
+      <c r="G17" s="38" t="str">
         <f aca="false">IF(E17="","",E17-IF(F17="",0,F17))</f>
         <v/>
       </c>
-      <c r="H17" s="19" t="str">
+      <c r="H17" s="38" t="str">
         <f aca="false">IF(A17="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C17,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I17" s="19" t="str">
+      <c r="I17" s="38" t="str">
         <f aca="false">IF(OR(G17="",H17=""),"",G17-H17)</f>
         <v/>
       </c>
-      <c r="J17" s="46" t="str">
+      <c r="J17" s="55" t="str">
         <f aca="false">IF(OR(I17="",H17="",H17=0),"",I17/H17)</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="47"/>
-      <c r="B18" s="22" t="str">
+      <c r="A18" s="56"/>
+      <c r="B18" s="41" t="str">
         <f aca="false">IF(A18="","",A18-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C18" s="22" t="str">
+      <c r="C18" s="41" t="str">
         <f aca="false">IF(A18="","",MIN(7,MAX(1,ROUNDUP(B18/7,0))))</f>
         <v/>
       </c>
-      <c r="D18" s="44" t="str">
+      <c r="D18" s="53" t="str">
         <f aca="false">IF(A18="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C18,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E18" s="48"/>
-      <c r="F18" s="48"/>
-      <c r="G18" s="19" t="str">
+      <c r="E18" s="57"/>
+      <c r="F18" s="57"/>
+      <c r="G18" s="38" t="str">
         <f aca="false">IF(E18="","",E18-IF(F18="",0,F18))</f>
         <v/>
       </c>
-      <c r="H18" s="19" t="str">
+      <c r="H18" s="38" t="str">
         <f aca="false">IF(A18="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C18,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I18" s="19" t="str">
+      <c r="I18" s="38" t="str">
         <f aca="false">IF(OR(G18="",H18=""),"",G18-H18)</f>
         <v/>
       </c>
-      <c r="J18" s="46" t="str">
+      <c r="J18" s="55" t="str">
         <f aca="false">IF(OR(I18="",H18="",H18=0),"",I18/H18)</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="47"/>
-      <c r="B19" s="22" t="str">
+      <c r="A19" s="56"/>
+      <c r="B19" s="41" t="str">
         <f aca="false">IF(A19="","",A19-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C19" s="22" t="str">
+      <c r="C19" s="41" t="str">
         <f aca="false">IF(A19="","",MIN(7,MAX(1,ROUNDUP(B19/7,0))))</f>
         <v/>
       </c>
-      <c r="D19" s="44" t="str">
+      <c r="D19" s="53" t="str">
         <f aca="false">IF(A19="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C19,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E19" s="48"/>
-      <c r="F19" s="48"/>
-      <c r="G19" s="19" t="str">
+      <c r="E19" s="57"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="38" t="str">
         <f aca="false">IF(E19="","",E19-IF(F19="",0,F19))</f>
         <v/>
       </c>
-      <c r="H19" s="19" t="str">
+      <c r="H19" s="38" t="str">
         <f aca="false">IF(A19="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C19,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I19" s="19" t="str">
+      <c r="I19" s="38" t="str">
         <f aca="false">IF(OR(G19="",H19=""),"",G19-H19)</f>
         <v/>
       </c>
-      <c r="J19" s="46" t="str">
+      <c r="J19" s="55" t="str">
         <f aca="false">IF(OR(I19="",H19="",H19=0),"",I19/H19)</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="47"/>
-      <c r="B20" s="22" t="str">
+      <c r="A20" s="56"/>
+      <c r="B20" s="41" t="str">
         <f aca="false">IF(A20="","",A20-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C20" s="22" t="str">
+      <c r="C20" s="41" t="str">
         <f aca="false">IF(A20="","",MIN(7,MAX(1,ROUNDUP(B20/7,0))))</f>
         <v/>
       </c>
-      <c r="D20" s="44" t="str">
+      <c r="D20" s="53" t="str">
         <f aca="false">IF(A20="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C20,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E20" s="48"/>
-      <c r="F20" s="48"/>
-      <c r="G20" s="19" t="str">
+      <c r="E20" s="57"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="38" t="str">
         <f aca="false">IF(E20="","",E20-IF(F20="",0,F20))</f>
         <v/>
       </c>
-      <c r="H20" s="19" t="str">
+      <c r="H20" s="38" t="str">
         <f aca="false">IF(A20="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C20,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I20" s="19" t="str">
+      <c r="I20" s="38" t="str">
         <f aca="false">IF(OR(G20="",H20=""),"",G20-H20)</f>
         <v/>
       </c>
-      <c r="J20" s="46" t="str">
+      <c r="J20" s="55" t="str">
         <f aca="false">IF(OR(I20="",H20="",H20=0),"",I20/H20)</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="47"/>
-      <c r="B21" s="22" t="str">
+      <c r="A21" s="56"/>
+      <c r="B21" s="41" t="str">
         <f aca="false">IF(A21="","",A21-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C21" s="22" t="str">
+      <c r="C21" s="41" t="str">
         <f aca="false">IF(A21="","",MIN(7,MAX(1,ROUNDUP(B21/7,0))))</f>
         <v/>
       </c>
-      <c r="D21" s="44" t="str">
+      <c r="D21" s="53" t="str">
         <f aca="false">IF(A21="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C21,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E21" s="48"/>
-      <c r="F21" s="48"/>
-      <c r="G21" s="19" t="str">
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="38" t="str">
         <f aca="false">IF(E21="","",E21-IF(F21="",0,F21))</f>
         <v/>
       </c>
-      <c r="H21" s="19" t="str">
+      <c r="H21" s="38" t="str">
         <f aca="false">IF(A21="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C21,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I21" s="19" t="str">
+      <c r="I21" s="38" t="str">
         <f aca="false">IF(OR(G21="",H21=""),"",G21-H21)</f>
         <v/>
       </c>
-      <c r="J21" s="46" t="str">
+      <c r="J21" s="55" t="str">
         <f aca="false">IF(OR(I21="",H21="",H21=0),"",I21/H21)</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="47"/>
-      <c r="B22" s="22" t="str">
+      <c r="A22" s="56"/>
+      <c r="B22" s="41" t="str">
         <f aca="false">IF(A22="","",A22-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C22" s="22" t="str">
+      <c r="C22" s="41" t="str">
         <f aca="false">IF(A22="","",MIN(7,MAX(1,ROUNDUP(B22/7,0))))</f>
         <v/>
       </c>
-      <c r="D22" s="44" t="str">
+      <c r="D22" s="53" t="str">
         <f aca="false">IF(A22="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C22,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E22" s="48"/>
-      <c r="F22" s="48"/>
-      <c r="G22" s="19" t="str">
+      <c r="E22" s="57"/>
+      <c r="F22" s="57"/>
+      <c r="G22" s="38" t="str">
         <f aca="false">IF(E22="","",E22-IF(F22="",0,F22))</f>
         <v/>
       </c>
-      <c r="H22" s="19" t="str">
+      <c r="H22" s="38" t="str">
         <f aca="false">IF(A22="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C22,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I22" s="19" t="str">
+      <c r="I22" s="38" t="str">
         <f aca="false">IF(OR(G22="",H22=""),"",G22-H22)</f>
         <v/>
       </c>
-      <c r="J22" s="46" t="str">
+      <c r="J22" s="55" t="str">
         <f aca="false">IF(OR(I22="",H22="",H22=0),"",I22/H22)</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="47"/>
-      <c r="B23" s="22" t="str">
+      <c r="A23" s="56"/>
+      <c r="B23" s="41" t="str">
         <f aca="false">IF(A23="","",A23-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C23" s="22" t="str">
+      <c r="C23" s="41" t="str">
         <f aca="false">IF(A23="","",MIN(7,MAX(1,ROUNDUP(B23/7,0))))</f>
         <v/>
       </c>
-      <c r="D23" s="44" t="str">
+      <c r="D23" s="53" t="str">
         <f aca="false">IF(A23="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C23,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E23" s="48"/>
-      <c r="F23" s="48"/>
-      <c r="G23" s="19" t="str">
+      <c r="E23" s="57"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="38" t="str">
         <f aca="false">IF(E23="","",E23-IF(F23="",0,F23))</f>
         <v/>
       </c>
-      <c r="H23" s="19" t="str">
+      <c r="H23" s="38" t="str">
         <f aca="false">IF(A23="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C23,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I23" s="19" t="str">
+      <c r="I23" s="38" t="str">
         <f aca="false">IF(OR(G23="",H23=""),"",G23-H23)</f>
         <v/>
       </c>
-      <c r="J23" s="46" t="str">
+      <c r="J23" s="55" t="str">
         <f aca="false">IF(OR(I23="",H23="",H23=0),"",I23/H23)</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="47"/>
-      <c r="B24" s="22" t="str">
+      <c r="A24" s="56"/>
+      <c r="B24" s="41" t="str">
         <f aca="false">IF(A24="","",A24-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C24" s="22" t="str">
+      <c r="C24" s="41" t="str">
         <f aca="false">IF(A24="","",MIN(7,MAX(1,ROUNDUP(B24/7,0))))</f>
         <v/>
       </c>
-      <c r="D24" s="44" t="str">
+      <c r="D24" s="53" t="str">
         <f aca="false">IF(A24="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C24,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E24" s="48"/>
-      <c r="F24" s="48"/>
-      <c r="G24" s="19" t="str">
+      <c r="E24" s="57"/>
+      <c r="F24" s="57"/>
+      <c r="G24" s="38" t="str">
         <f aca="false">IF(E24="","",E24-IF(F24="",0,F24))</f>
         <v/>
       </c>
-      <c r="H24" s="19" t="str">
+      <c r="H24" s="38" t="str">
         <f aca="false">IF(A24="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C24,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I24" s="19" t="str">
+      <c r="I24" s="38" t="str">
         <f aca="false">IF(OR(G24="",H24=""),"",G24-H24)</f>
         <v/>
       </c>
-      <c r="J24" s="46" t="str">
+      <c r="J24" s="55" t="str">
         <f aca="false">IF(OR(I24="",H24="",H24=0),"",I24/H24)</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="47"/>
-      <c r="B25" s="22" t="str">
+      <c r="A25" s="56"/>
+      <c r="B25" s="41" t="str">
         <f aca="false">IF(A25="","",A25-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C25" s="22" t="str">
+      <c r="C25" s="41" t="str">
         <f aca="false">IF(A25="","",MIN(7,MAX(1,ROUNDUP(B25/7,0))))</f>
         <v/>
       </c>
-      <c r="D25" s="44" t="str">
+      <c r="D25" s="53" t="str">
         <f aca="false">IF(A25="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C25,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E25" s="48"/>
-      <c r="F25" s="48"/>
-      <c r="G25" s="19" t="str">
+      <c r="E25" s="57"/>
+      <c r="F25" s="57"/>
+      <c r="G25" s="38" t="str">
         <f aca="false">IF(E25="","",E25-IF(F25="",0,F25))</f>
         <v/>
       </c>
-      <c r="H25" s="19" t="str">
+      <c r="H25" s="38" t="str">
         <f aca="false">IF(A25="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C25,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I25" s="19" t="str">
+      <c r="I25" s="38" t="str">
         <f aca="false">IF(OR(G25="",H25=""),"",G25-H25)</f>
         <v/>
       </c>
-      <c r="J25" s="46" t="str">
+      <c r="J25" s="55" t="str">
         <f aca="false">IF(OR(I25="",H25="",H25=0),"",I25/H25)</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="47"/>
-      <c r="B26" s="22" t="str">
+      <c r="A26" s="56"/>
+      <c r="B26" s="41" t="str">
         <f aca="false">IF(A26="","",A26-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C26" s="22" t="str">
+      <c r="C26" s="41" t="str">
         <f aca="false">IF(A26="","",MIN(7,MAX(1,ROUNDUP(B26/7,0))))</f>
         <v/>
       </c>
-      <c r="D26" s="44" t="str">
+      <c r="D26" s="53" t="str">
         <f aca="false">IF(A26="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C26,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E26" s="48"/>
-      <c r="F26" s="48"/>
-      <c r="G26" s="19" t="str">
+      <c r="E26" s="57"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="38" t="str">
         <f aca="false">IF(E26="","",E26-IF(F26="",0,F26))</f>
         <v/>
       </c>
-      <c r="H26" s="19" t="str">
+      <c r="H26" s="38" t="str">
         <f aca="false">IF(A26="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C26,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I26" s="19" t="str">
+      <c r="I26" s="38" t="str">
         <f aca="false">IF(OR(G26="",H26=""),"",G26-H26)</f>
         <v/>
       </c>
-      <c r="J26" s="46" t="str">
+      <c r="J26" s="55" t="str">
         <f aca="false">IF(OR(I26="",H26="",H26=0),"",I26/H26)</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="47"/>
-      <c r="B27" s="22" t="str">
+      <c r="A27" s="56"/>
+      <c r="B27" s="41" t="str">
         <f aca="false">IF(A27="","",A27-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C27" s="22" t="str">
+      <c r="C27" s="41" t="str">
         <f aca="false">IF(A27="","",MIN(7,MAX(1,ROUNDUP(B27/7,0))))</f>
         <v/>
       </c>
-      <c r="D27" s="44" t="str">
+      <c r="D27" s="53" t="str">
         <f aca="false">IF(A27="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C27,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E27" s="48"/>
-      <c r="F27" s="48"/>
-      <c r="G27" s="19" t="str">
+      <c r="E27" s="57"/>
+      <c r="F27" s="57"/>
+      <c r="G27" s="38" t="str">
         <f aca="false">IF(E27="","",E27-IF(F27="",0,F27))</f>
         <v/>
       </c>
-      <c r="H27" s="19" t="str">
+      <c r="H27" s="38" t="str">
         <f aca="false">IF(A27="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C27,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I27" s="19" t="str">
+      <c r="I27" s="38" t="str">
         <f aca="false">IF(OR(G27="",H27=""),"",G27-H27)</f>
         <v/>
       </c>
-      <c r="J27" s="46" t="str">
+      <c r="J27" s="55" t="str">
         <f aca="false">IF(OR(I27="",H27="",H27=0),"",I27/H27)</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="47"/>
-      <c r="B28" s="22" t="str">
+      <c r="A28" s="56"/>
+      <c r="B28" s="41" t="str">
         <f aca="false">IF(A28="","",A28-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C28" s="22" t="str">
+      <c r="C28" s="41" t="str">
         <f aca="false">IF(A28="","",MIN(7,MAX(1,ROUNDUP(B28/7,0))))</f>
         <v/>
       </c>
-      <c r="D28" s="44" t="str">
+      <c r="D28" s="53" t="str">
         <f aca="false">IF(A28="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C28,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E28" s="48"/>
-      <c r="F28" s="48"/>
-      <c r="G28" s="19" t="str">
+      <c r="E28" s="57"/>
+      <c r="F28" s="57"/>
+      <c r="G28" s="38" t="str">
         <f aca="false">IF(E28="","",E28-IF(F28="",0,F28))</f>
         <v/>
       </c>
-      <c r="H28" s="19" t="str">
+      <c r="H28" s="38" t="str">
         <f aca="false">IF(A28="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C28,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I28" s="19" t="str">
+      <c r="I28" s="38" t="str">
         <f aca="false">IF(OR(G28="",H28=""),"",G28-H28)</f>
         <v/>
       </c>
-      <c r="J28" s="46" t="str">
+      <c r="J28" s="55" t="str">
         <f aca="false">IF(OR(I28="",H28="",H28=0),"",I28/H28)</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="47"/>
-      <c r="B29" s="22" t="str">
+      <c r="A29" s="56"/>
+      <c r="B29" s="41" t="str">
         <f aca="false">IF(A29="","",A29-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C29" s="22" t="str">
+      <c r="C29" s="41" t="str">
         <f aca="false">IF(A29="","",MIN(7,MAX(1,ROUNDUP(B29/7,0))))</f>
         <v/>
       </c>
-      <c r="D29" s="44" t="str">
+      <c r="D29" s="53" t="str">
         <f aca="false">IF(A29="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C29,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E29" s="48"/>
-      <c r="F29" s="48"/>
-      <c r="G29" s="19" t="str">
+      <c r="E29" s="57"/>
+      <c r="F29" s="57"/>
+      <c r="G29" s="38" t="str">
         <f aca="false">IF(E29="","",E29-IF(F29="",0,F29))</f>
         <v/>
       </c>
-      <c r="H29" s="19" t="str">
+      <c r="H29" s="38" t="str">
         <f aca="false">IF(A29="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C29,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I29" s="19" t="str">
+      <c r="I29" s="38" t="str">
         <f aca="false">IF(OR(G29="",H29=""),"",G29-H29)</f>
         <v/>
       </c>
-      <c r="J29" s="46" t="str">
+      <c r="J29" s="55" t="str">
         <f aca="false">IF(OR(I29="",H29="",H29=0),"",I29/H29)</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="47"/>
-      <c r="B30" s="22" t="str">
+      <c r="A30" s="56"/>
+      <c r="B30" s="41" t="str">
         <f aca="false">IF(A30="","",A30-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C30" s="22" t="str">
+      <c r="C30" s="41" t="str">
         <f aca="false">IF(A30="","",MIN(7,MAX(1,ROUNDUP(B30/7,0))))</f>
         <v/>
       </c>
-      <c r="D30" s="44" t="str">
+      <c r="D30" s="53" t="str">
         <f aca="false">IF(A30="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C30,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E30" s="48"/>
-      <c r="F30" s="48"/>
-      <c r="G30" s="19" t="str">
+      <c r="E30" s="57"/>
+      <c r="F30" s="57"/>
+      <c r="G30" s="38" t="str">
         <f aca="false">IF(E30="","",E30-IF(F30="",0,F30))</f>
         <v/>
       </c>
-      <c r="H30" s="19" t="str">
+      <c r="H30" s="38" t="str">
         <f aca="false">IF(A30="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C30,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I30" s="19" t="str">
+      <c r="I30" s="38" t="str">
         <f aca="false">IF(OR(G30="",H30=""),"",G30-H30)</f>
         <v/>
       </c>
-      <c r="J30" s="46" t="str">
+      <c r="J30" s="55" t="str">
         <f aca="false">IF(OR(I30="",H30="",H30=0),"",I30/H30)</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="47"/>
-      <c r="B31" s="22" t="str">
+      <c r="A31" s="56"/>
+      <c r="B31" s="41" t="str">
         <f aca="false">IF(A31="","",A31-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C31" s="22" t="str">
+      <c r="C31" s="41" t="str">
         <f aca="false">IF(A31="","",MIN(7,MAX(1,ROUNDUP(B31/7,0))))</f>
         <v/>
       </c>
-      <c r="D31" s="44" t="str">
+      <c r="D31" s="53" t="str">
         <f aca="false">IF(A31="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C31,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E31" s="48"/>
-      <c r="F31" s="48"/>
-      <c r="G31" s="19" t="str">
+      <c r="E31" s="57"/>
+      <c r="F31" s="57"/>
+      <c r="G31" s="38" t="str">
         <f aca="false">IF(E31="","",E31-IF(F31="",0,F31))</f>
         <v/>
       </c>
-      <c r="H31" s="19" t="str">
+      <c r="H31" s="38" t="str">
         <f aca="false">IF(A31="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C31,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I31" s="19" t="str">
+      <c r="I31" s="38" t="str">
         <f aca="false">IF(OR(G31="",H31=""),"",G31-H31)</f>
         <v/>
       </c>
-      <c r="J31" s="46" t="str">
+      <c r="J31" s="55" t="str">
         <f aca="false">IF(OR(I31="",H31="",H31=0),"",I31/H31)</f>
         <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="47"/>
-      <c r="B32" s="22" t="str">
+      <c r="A32" s="56"/>
+      <c r="B32" s="41" t="str">
         <f aca="false">IF(A32="","",A32-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C32" s="22" t="str">
+      <c r="C32" s="41" t="str">
         <f aca="false">IF(A32="","",MIN(7,MAX(1,ROUNDUP(B32/7,0))))</f>
         <v/>
       </c>
-      <c r="D32" s="44" t="str">
+      <c r="D32" s="53" t="str">
         <f aca="false">IF(A32="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C32,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E32" s="48"/>
-      <c r="F32" s="48"/>
-      <c r="G32" s="19" t="str">
+      <c r="E32" s="57"/>
+      <c r="F32" s="57"/>
+      <c r="G32" s="38" t="str">
         <f aca="false">IF(E32="","",E32-IF(F32="",0,F32))</f>
         <v/>
       </c>
-      <c r="H32" s="19" t="str">
+      <c r="H32" s="38" t="str">
         <f aca="false">IF(A32="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C32,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I32" s="19" t="str">
+      <c r="I32" s="38" t="str">
         <f aca="false">IF(OR(G32="",H32=""),"",G32-H32)</f>
         <v/>
       </c>
-      <c r="J32" s="46" t="str">
+      <c r="J32" s="55" t="str">
         <f aca="false">IF(OR(I32="",H32="",H32=0),"",I32/H32)</f>
         <v/>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="47"/>
-      <c r="B33" s="22" t="str">
+      <c r="A33" s="56"/>
+      <c r="B33" s="41" t="str">
         <f aca="false">IF(A33="","",A33-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C33" s="22" t="str">
+      <c r="C33" s="41" t="str">
         <f aca="false">IF(A33="","",MIN(7,MAX(1,ROUNDUP(B33/7,0))))</f>
         <v/>
       </c>
-      <c r="D33" s="44" t="str">
+      <c r="D33" s="53" t="str">
         <f aca="false">IF(A33="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C33,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E33" s="48"/>
-      <c r="F33" s="48"/>
-      <c r="G33" s="19" t="str">
+      <c r="E33" s="57"/>
+      <c r="F33" s="57"/>
+      <c r="G33" s="38" t="str">
         <f aca="false">IF(E33="","",E33-IF(F33="",0,F33))</f>
         <v/>
       </c>
-      <c r="H33" s="19" t="str">
+      <c r="H33" s="38" t="str">
         <f aca="false">IF(A33="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C33,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I33" s="19" t="str">
+      <c r="I33" s="38" t="str">
         <f aca="false">IF(OR(G33="",H33=""),"",G33-H33)</f>
         <v/>
       </c>
-      <c r="J33" s="46" t="str">
+      <c r="J33" s="55" t="str">
         <f aca="false">IF(OR(I33="",H33="",H33=0),"",I33/H33)</f>
         <v/>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="47"/>
-      <c r="B34" s="22" t="str">
+      <c r="A34" s="56"/>
+      <c r="B34" s="41" t="str">
         <f aca="false">IF(A34="","",A34-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C34" s="22" t="str">
+      <c r="C34" s="41" t="str">
         <f aca="false">IF(A34="","",MIN(7,MAX(1,ROUNDUP(B34/7,0))))</f>
         <v/>
       </c>
-      <c r="D34" s="44" t="str">
+      <c r="D34" s="53" t="str">
         <f aca="false">IF(A34="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C34,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E34" s="48"/>
-      <c r="F34" s="48"/>
-      <c r="G34" s="19" t="str">
+      <c r="E34" s="57"/>
+      <c r="F34" s="57"/>
+      <c r="G34" s="38" t="str">
         <f aca="false">IF(E34="","",E34-IF(F34="",0,F34))</f>
         <v/>
       </c>
-      <c r="H34" s="19" t="str">
+      <c r="H34" s="38" t="str">
         <f aca="false">IF(A34="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C34,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I34" s="19" t="str">
+      <c r="I34" s="38" t="str">
         <f aca="false">IF(OR(G34="",H34=""),"",G34-H34)</f>
         <v/>
       </c>
-      <c r="J34" s="46" t="str">
+      <c r="J34" s="55" t="str">
         <f aca="false">IF(OR(I34="",H34="",H34=0),"",I34/H34)</f>
         <v/>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="47"/>
-      <c r="B35" s="22" t="str">
+      <c r="A35" s="56"/>
+      <c r="B35" s="41" t="str">
         <f aca="false">IF(A35="","",A35-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C35" s="22" t="str">
+      <c r="C35" s="41" t="str">
         <f aca="false">IF(A35="","",MIN(7,MAX(1,ROUNDUP(B35/7,0))))</f>
         <v/>
       </c>
-      <c r="D35" s="44" t="str">
+      <c r="D35" s="53" t="str">
         <f aca="false">IF(A35="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C35,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E35" s="48"/>
-      <c r="F35" s="48"/>
-      <c r="G35" s="19" t="str">
+      <c r="E35" s="57"/>
+      <c r="F35" s="57"/>
+      <c r="G35" s="38" t="str">
         <f aca="false">IF(E35="","",E35-IF(F35="",0,F35))</f>
         <v/>
       </c>
-      <c r="H35" s="19" t="str">
+      <c r="H35" s="38" t="str">
         <f aca="false">IF(A35="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C35,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I35" s="19" t="str">
+      <c r="I35" s="38" t="str">
         <f aca="false">IF(OR(G35="",H35=""),"",G35-H35)</f>
         <v/>
       </c>
-      <c r="J35" s="46" t="str">
+      <c r="J35" s="55" t="str">
         <f aca="false">IF(OR(I35="",H35="",H35=0),"",I35/H35)</f>
         <v/>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="47"/>
-      <c r="B36" s="22" t="str">
+      <c r="A36" s="56"/>
+      <c r="B36" s="41" t="str">
         <f aca="false">IF(A36="","",A36-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C36" s="22" t="str">
+      <c r="C36" s="41" t="str">
         <f aca="false">IF(A36="","",MIN(7,MAX(1,ROUNDUP(B36/7,0))))</f>
         <v/>
       </c>
-      <c r="D36" s="44" t="str">
+      <c r="D36" s="53" t="str">
         <f aca="false">IF(A36="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C36,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E36" s="48"/>
-      <c r="F36" s="48"/>
-      <c r="G36" s="19" t="str">
+      <c r="E36" s="57"/>
+      <c r="F36" s="57"/>
+      <c r="G36" s="38" t="str">
         <f aca="false">IF(E36="","",E36-IF(F36="",0,F36))</f>
         <v/>
       </c>
-      <c r="H36" s="19" t="str">
+      <c r="H36" s="38" t="str">
         <f aca="false">IF(A36="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C36,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I36" s="19" t="str">
+      <c r="I36" s="38" t="str">
         <f aca="false">IF(OR(G36="",H36=""),"",G36-H36)</f>
         <v/>
       </c>
-      <c r="J36" s="46" t="str">
+      <c r="J36" s="55" t="str">
         <f aca="false">IF(OR(I36="",H36="",H36=0),"",I36/H36)</f>
         <v/>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="47"/>
-      <c r="B37" s="22" t="str">
+      <c r="A37" s="56"/>
+      <c r="B37" s="41" t="str">
         <f aca="false">IF(A37="","",A37-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C37" s="22" t="str">
+      <c r="C37" s="41" t="str">
         <f aca="false">IF(A37="","",MIN(7,MAX(1,ROUNDUP(B37/7,0))))</f>
         <v/>
       </c>
-      <c r="D37" s="44" t="str">
+      <c r="D37" s="53" t="str">
         <f aca="false">IF(A37="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C37,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E37" s="48"/>
-      <c r="F37" s="48"/>
-      <c r="G37" s="19" t="str">
+      <c r="E37" s="57"/>
+      <c r="F37" s="57"/>
+      <c r="G37" s="38" t="str">
         <f aca="false">IF(E37="","",E37-IF(F37="",0,F37))</f>
         <v/>
       </c>
-      <c r="H37" s="19" t="str">
+      <c r="H37" s="38" t="str">
         <f aca="false">IF(A37="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C37,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I37" s="19" t="str">
+      <c r="I37" s="38" t="str">
         <f aca="false">IF(OR(G37="",H37=""),"",G37-H37)</f>
         <v/>
       </c>
-      <c r="J37" s="46" t="str">
+      <c r="J37" s="55" t="str">
         <f aca="false">IF(OR(I37="",H37="",H37=0),"",I37/H37)</f>
         <v/>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="47"/>
-      <c r="B38" s="22" t="str">
+      <c r="A38" s="56"/>
+      <c r="B38" s="41" t="str">
         <f aca="false">IF(A38="","",A38-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C38" s="22" t="str">
+      <c r="C38" s="41" t="str">
         <f aca="false">IF(A38="","",MIN(7,MAX(1,ROUNDUP(B38/7,0))))</f>
         <v/>
       </c>
-      <c r="D38" s="44" t="str">
+      <c r="D38" s="53" t="str">
         <f aca="false">IF(A38="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C38,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E38" s="48"/>
-      <c r="F38" s="48"/>
-      <c r="G38" s="19" t="str">
+      <c r="E38" s="57"/>
+      <c r="F38" s="57"/>
+      <c r="G38" s="38" t="str">
         <f aca="false">IF(E38="","",E38-IF(F38="",0,F38))</f>
         <v/>
       </c>
-      <c r="H38" s="19" t="str">
+      <c r="H38" s="38" t="str">
         <f aca="false">IF(A38="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C38,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I38" s="19" t="str">
+      <c r="I38" s="38" t="str">
         <f aca="false">IF(OR(G38="",H38=""),"",G38-H38)</f>
         <v/>
       </c>
-      <c r="J38" s="46" t="str">
+      <c r="J38" s="55" t="str">
         <f aca="false">IF(OR(I38="",H38="",H38=0),"",I38/H38)</f>
         <v/>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="47"/>
-      <c r="B39" s="22" t="str">
+      <c r="A39" s="56"/>
+      <c r="B39" s="41" t="str">
         <f aca="false">IF(A39="","",A39-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C39" s="22" t="str">
+      <c r="C39" s="41" t="str">
         <f aca="false">IF(A39="","",MIN(7,MAX(1,ROUNDUP(B39/7,0))))</f>
         <v/>
       </c>
-      <c r="D39" s="44" t="str">
+      <c r="D39" s="53" t="str">
         <f aca="false">IF(A39="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C39,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E39" s="48"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="19" t="str">
+      <c r="E39" s="57"/>
+      <c r="F39" s="57"/>
+      <c r="G39" s="38" t="str">
         <f aca="false">IF(E39="","",E39-IF(F39="",0,F39))</f>
         <v/>
       </c>
-      <c r="H39" s="19" t="str">
+      <c r="H39" s="38" t="str">
         <f aca="false">IF(A39="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C39,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I39" s="19" t="str">
+      <c r="I39" s="38" t="str">
         <f aca="false">IF(OR(G39="",H39=""),"",G39-H39)</f>
         <v/>
       </c>
-      <c r="J39" s="46" t="str">
+      <c r="J39" s="55" t="str">
         <f aca="false">IF(OR(I39="",H39="",H39=0),"",I39/H39)</f>
         <v/>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="47"/>
-      <c r="B40" s="22" t="str">
+      <c r="A40" s="56"/>
+      <c r="B40" s="41" t="str">
         <f aca="false">IF(A40="","",A40-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C40" s="22" t="str">
+      <c r="C40" s="41" t="str">
         <f aca="false">IF(A40="","",MIN(7,MAX(1,ROUNDUP(B40/7,0))))</f>
         <v/>
       </c>
-      <c r="D40" s="44" t="str">
+      <c r="D40" s="53" t="str">
         <f aca="false">IF(A40="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C40,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="19" t="str">
+      <c r="E40" s="57"/>
+      <c r="F40" s="57"/>
+      <c r="G40" s="38" t="str">
         <f aca="false">IF(E40="","",E40-IF(F40="",0,F40))</f>
         <v/>
       </c>
-      <c r="H40" s="19" t="str">
+      <c r="H40" s="38" t="str">
         <f aca="false">IF(A40="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C40,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I40" s="19" t="str">
+      <c r="I40" s="38" t="str">
         <f aca="false">IF(OR(G40="",H40=""),"",G40-H40)</f>
         <v/>
       </c>
-      <c r="J40" s="46" t="str">
+      <c r="J40" s="55" t="str">
         <f aca="false">IF(OR(I40="",H40="",H40=0),"",I40/H40)</f>
         <v/>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="47"/>
-      <c r="B41" s="22" t="str">
+      <c r="A41" s="56"/>
+      <c r="B41" s="41" t="str">
         <f aca="false">IF(A41="","",A41-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C41" s="22" t="str">
+      <c r="C41" s="41" t="str">
         <f aca="false">IF(A41="","",MIN(7,MAX(1,ROUNDUP(B41/7,0))))</f>
         <v/>
       </c>
-      <c r="D41" s="44" t="str">
+      <c r="D41" s="53" t="str">
         <f aca="false">IF(A41="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C41,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E41" s="48"/>
-      <c r="F41" s="48"/>
-      <c r="G41" s="19" t="str">
+      <c r="E41" s="57"/>
+      <c r="F41" s="57"/>
+      <c r="G41" s="38" t="str">
         <f aca="false">IF(E41="","",E41-IF(F41="",0,F41))</f>
         <v/>
       </c>
-      <c r="H41" s="19" t="str">
+      <c r="H41" s="38" t="str">
         <f aca="false">IF(A41="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C41,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I41" s="19" t="str">
+      <c r="I41" s="38" t="str">
         <f aca="false">IF(OR(G41="",H41=""),"",G41-H41)</f>
         <v/>
       </c>
-      <c r="J41" s="46" t="str">
+      <c r="J41" s="55" t="str">
         <f aca="false">IF(OR(I41="",H41="",H41=0),"",I41/H41)</f>
         <v/>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="47"/>
-      <c r="B42" s="22" t="str">
+      <c r="A42" s="56"/>
+      <c r="B42" s="41" t="str">
         <f aca="false">IF(A42="","",A42-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C42" s="22" t="str">
+      <c r="C42" s="41" t="str">
         <f aca="false">IF(A42="","",MIN(7,MAX(1,ROUNDUP(B42/7,0))))</f>
         <v/>
       </c>
-      <c r="D42" s="44" t="str">
+      <c r="D42" s="53" t="str">
         <f aca="false">IF(A42="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C42,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E42" s="48"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="19" t="str">
+      <c r="E42" s="57"/>
+      <c r="F42" s="57"/>
+      <c r="G42" s="38" t="str">
         <f aca="false">IF(E42="","",E42-IF(F42="",0,F42))</f>
         <v/>
       </c>
-      <c r="H42" s="19" t="str">
+      <c r="H42" s="38" t="str">
         <f aca="false">IF(A42="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C42,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I42" s="19" t="str">
+      <c r="I42" s="38" t="str">
         <f aca="false">IF(OR(G42="",H42=""),"",G42-H42)</f>
         <v/>
       </c>
-      <c r="J42" s="46" t="str">
+      <c r="J42" s="55" t="str">
         <f aca="false">IF(OR(I42="",H42="",H42=0),"",I42/H42)</f>
         <v/>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="47"/>
-      <c r="B43" s="22" t="str">
+      <c r="A43" s="56"/>
+      <c r="B43" s="41" t="str">
         <f aca="false">IF(A43="","",A43-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C43" s="22" t="str">
+      <c r="C43" s="41" t="str">
         <f aca="false">IF(A43="","",MIN(7,MAX(1,ROUNDUP(B43/7,0))))</f>
         <v/>
       </c>
-      <c r="D43" s="44" t="str">
+      <c r="D43" s="53" t="str">
         <f aca="false">IF(A43="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C43,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E43" s="48"/>
-      <c r="F43" s="48"/>
-      <c r="G43" s="19" t="str">
+      <c r="E43" s="57"/>
+      <c r="F43" s="57"/>
+      <c r="G43" s="38" t="str">
         <f aca="false">IF(E43="","",E43-IF(F43="",0,F43))</f>
         <v/>
       </c>
-      <c r="H43" s="19" t="str">
+      <c r="H43" s="38" t="str">
         <f aca="false">IF(A43="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C43,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I43" s="19" t="str">
+      <c r="I43" s="38" t="str">
         <f aca="false">IF(OR(G43="",H43=""),"",G43-H43)</f>
         <v/>
       </c>
-      <c r="J43" s="46" t="str">
+      <c r="J43" s="55" t="str">
         <f aca="false">IF(OR(I43="",H43="",H43=0),"",I43/H43)</f>
         <v/>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="47"/>
-      <c r="B44" s="22" t="str">
+      <c r="A44" s="56"/>
+      <c r="B44" s="41" t="str">
         <f aca="false">IF(A44="","",A44-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C44" s="22" t="str">
+      <c r="C44" s="41" t="str">
         <f aca="false">IF(A44="","",MIN(7,MAX(1,ROUNDUP(B44/7,0))))</f>
         <v/>
       </c>
-      <c r="D44" s="44" t="str">
+      <c r="D44" s="53" t="str">
         <f aca="false">IF(A44="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C44,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E44" s="48"/>
-      <c r="F44" s="48"/>
-      <c r="G44" s="19" t="str">
+      <c r="E44" s="57"/>
+      <c r="F44" s="57"/>
+      <c r="G44" s="38" t="str">
         <f aca="false">IF(E44="","",E44-IF(F44="",0,F44))</f>
         <v/>
       </c>
-      <c r="H44" s="19" t="str">
+      <c r="H44" s="38" t="str">
         <f aca="false">IF(A44="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C44,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I44" s="19" t="str">
+      <c r="I44" s="38" t="str">
         <f aca="false">IF(OR(G44="",H44=""),"",G44-H44)</f>
         <v/>
       </c>
-      <c r="J44" s="46" t="str">
+      <c r="J44" s="55" t="str">
         <f aca="false">IF(OR(I44="",H44="",H44=0),"",I44/H44)</f>
         <v/>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="47"/>
-      <c r="B45" s="22" t="str">
+      <c r="A45" s="56"/>
+      <c r="B45" s="41" t="str">
         <f aca="false">IF(A45="","",A45-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C45" s="22" t="str">
+      <c r="C45" s="41" t="str">
         <f aca="false">IF(A45="","",MIN(7,MAX(1,ROUNDUP(B45/7,0))))</f>
         <v/>
       </c>
-      <c r="D45" s="44" t="str">
+      <c r="D45" s="53" t="str">
         <f aca="false">IF(A45="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C45,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E45" s="48"/>
-      <c r="F45" s="48"/>
-      <c r="G45" s="19" t="str">
+      <c r="E45" s="57"/>
+      <c r="F45" s="57"/>
+      <c r="G45" s="38" t="str">
         <f aca="false">IF(E45="","",E45-IF(F45="",0,F45))</f>
         <v/>
       </c>
-      <c r="H45" s="19" t="str">
+      <c r="H45" s="38" t="str">
         <f aca="false">IF(A45="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C45,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I45" s="19" t="str">
+      <c r="I45" s="38" t="str">
         <f aca="false">IF(OR(G45="",H45=""),"",G45-H45)</f>
         <v/>
       </c>
-      <c r="J45" s="46" t="str">
+      <c r="J45" s="55" t="str">
         <f aca="false">IF(OR(I45="",H45="",H45=0),"",I45/H45)</f>
         <v/>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="47"/>
-      <c r="B46" s="22" t="str">
+      <c r="A46" s="56"/>
+      <c r="B46" s="41" t="str">
         <f aca="false">IF(A46="","",A46-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C46" s="22" t="str">
+      <c r="C46" s="41" t="str">
         <f aca="false">IF(A46="","",MIN(7,MAX(1,ROUNDUP(B46/7,0))))</f>
         <v/>
       </c>
-      <c r="D46" s="44" t="str">
+      <c r="D46" s="53" t="str">
         <f aca="false">IF(A46="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C46,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E46" s="48"/>
-      <c r="F46" s="48"/>
-      <c r="G46" s="19" t="str">
+      <c r="E46" s="57"/>
+      <c r="F46" s="57"/>
+      <c r="G46" s="38" t="str">
         <f aca="false">IF(E46="","",E46-IF(F46="",0,F46))</f>
         <v/>
       </c>
-      <c r="H46" s="19" t="str">
+      <c r="H46" s="38" t="str">
         <f aca="false">IF(A46="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C46,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I46" s="19" t="str">
+      <c r="I46" s="38" t="str">
         <f aca="false">IF(OR(G46="",H46=""),"",G46-H46)</f>
         <v/>
       </c>
-      <c r="J46" s="46" t="str">
+      <c r="J46" s="55" t="str">
         <f aca="false">IF(OR(I46="",H46="",H46=0),"",I46/H46)</f>
         <v/>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="47"/>
-      <c r="B47" s="22" t="str">
+      <c r="A47" s="56"/>
+      <c r="B47" s="41" t="str">
         <f aca="false">IF(A47="","",A47-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C47" s="22" t="str">
+      <c r="C47" s="41" t="str">
         <f aca="false">IF(A47="","",MIN(7,MAX(1,ROUNDUP(B47/7,0))))</f>
         <v/>
       </c>
-      <c r="D47" s="44" t="str">
+      <c r="D47" s="53" t="str">
         <f aca="false">IF(A47="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C47,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E47" s="48"/>
-      <c r="F47" s="48"/>
-      <c r="G47" s="19" t="str">
+      <c r="E47" s="57"/>
+      <c r="F47" s="57"/>
+      <c r="G47" s="38" t="str">
         <f aca="false">IF(E47="","",E47-IF(F47="",0,F47))</f>
         <v/>
       </c>
-      <c r="H47" s="19" t="str">
+      <c r="H47" s="38" t="str">
         <f aca="false">IF(A47="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C47,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I47" s="19" t="str">
+      <c r="I47" s="38" t="str">
         <f aca="false">IF(OR(G47="",H47=""),"",G47-H47)</f>
         <v/>
       </c>
-      <c r="J47" s="46" t="str">
+      <c r="J47" s="55" t="str">
         <f aca="false">IF(OR(I47="",H47="",H47=0),"",I47/H47)</f>
         <v/>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="47"/>
-      <c r="B48" s="22" t="str">
+      <c r="A48" s="56"/>
+      <c r="B48" s="41" t="str">
         <f aca="false">IF(A48="","",A48-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C48" s="22" t="str">
+      <c r="C48" s="41" t="str">
         <f aca="false">IF(A48="","",MIN(7,MAX(1,ROUNDUP(B48/7,0))))</f>
         <v/>
       </c>
-      <c r="D48" s="44" t="str">
+      <c r="D48" s="53" t="str">
         <f aca="false">IF(A48="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C48,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E48" s="48"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="19" t="str">
+      <c r="E48" s="57"/>
+      <c r="F48" s="57"/>
+      <c r="G48" s="38" t="str">
         <f aca="false">IF(E48="","",E48-IF(F48="",0,F48))</f>
         <v/>
       </c>
-      <c r="H48" s="19" t="str">
+      <c r="H48" s="38" t="str">
         <f aca="false">IF(A48="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C48,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I48" s="19" t="str">
+      <c r="I48" s="38" t="str">
         <f aca="false">IF(OR(G48="",H48=""),"",G48-H48)</f>
         <v/>
       </c>
-      <c r="J48" s="46" t="str">
+      <c r="J48" s="55" t="str">
         <f aca="false">IF(OR(I48="",H48="",H48=0),"",I48/H48)</f>
         <v/>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="47"/>
-      <c r="B49" s="22" t="str">
+      <c r="A49" s="56"/>
+      <c r="B49" s="41" t="str">
         <f aca="false">IF(A49="","",A49-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C49" s="22" t="str">
+      <c r="C49" s="41" t="str">
         <f aca="false">IF(A49="","",MIN(7,MAX(1,ROUNDUP(B49/7,0))))</f>
         <v/>
       </c>
-      <c r="D49" s="44" t="str">
+      <c r="D49" s="53" t="str">
         <f aca="false">IF(A49="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C49,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E49" s="48"/>
-      <c r="F49" s="48"/>
-      <c r="G49" s="19" t="str">
+      <c r="E49" s="57"/>
+      <c r="F49" s="57"/>
+      <c r="G49" s="38" t="str">
         <f aca="false">IF(E49="","",E49-IF(F49="",0,F49))</f>
         <v/>
       </c>
-      <c r="H49" s="19" t="str">
+      <c r="H49" s="38" t="str">
         <f aca="false">IF(A49="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C49,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I49" s="19" t="str">
+      <c r="I49" s="38" t="str">
         <f aca="false">IF(OR(G49="",H49=""),"",G49-H49)</f>
         <v/>
       </c>
-      <c r="J49" s="46" t="str">
+      <c r="J49" s="55" t="str">
         <f aca="false">IF(OR(I49="",H49="",H49=0),"",I49/H49)</f>
         <v/>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="47"/>
-      <c r="B50" s="22" t="str">
+      <c r="A50" s="56"/>
+      <c r="B50" s="41" t="str">
         <f aca="false">IF(A50="","",A50-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C50" s="22" t="str">
+      <c r="C50" s="41" t="str">
         <f aca="false">IF(A50="","",MIN(7,MAX(1,ROUNDUP(B50/7,0))))</f>
         <v/>
       </c>
-      <c r="D50" s="44" t="str">
+      <c r="D50" s="53" t="str">
         <f aca="false">IF(A50="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C50,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E50" s="48"/>
-      <c r="F50" s="48"/>
-      <c r="G50" s="19" t="str">
+      <c r="E50" s="57"/>
+      <c r="F50" s="57"/>
+      <c r="G50" s="38" t="str">
         <f aca="false">IF(E50="","",E50-IF(F50="",0,F50))</f>
         <v/>
       </c>
-      <c r="H50" s="19" t="str">
+      <c r="H50" s="38" t="str">
         <f aca="false">IF(A50="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C50,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I50" s="19" t="str">
+      <c r="I50" s="38" t="str">
         <f aca="false">IF(OR(G50="",H50=""),"",G50-H50)</f>
         <v/>
       </c>
-      <c r="J50" s="46" t="str">
+      <c r="J50" s="55" t="str">
         <f aca="false">IF(OR(I50="",H50="",H50=0),"",I50/H50)</f>
         <v/>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="47"/>
-      <c r="B51" s="22" t="str">
+      <c r="A51" s="56"/>
+      <c r="B51" s="41" t="str">
         <f aca="false">IF(A51="","",A51-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C51" s="22" t="str">
+      <c r="C51" s="41" t="str">
         <f aca="false">IF(A51="","",MIN(7,MAX(1,ROUNDUP(B51/7,0))))</f>
         <v/>
       </c>
-      <c r="D51" s="44" t="str">
+      <c r="D51" s="53" t="str">
         <f aca="false">IF(A51="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C51,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E51" s="48"/>
-      <c r="F51" s="48"/>
-      <c r="G51" s="19" t="str">
+      <c r="E51" s="57"/>
+      <c r="F51" s="57"/>
+      <c r="G51" s="38" t="str">
         <f aca="false">IF(E51="","",E51-IF(F51="",0,F51))</f>
         <v/>
       </c>
-      <c r="H51" s="19" t="str">
+      <c r="H51" s="38" t="str">
         <f aca="false">IF(A51="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C51,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I51" s="19" t="str">
+      <c r="I51" s="38" t="str">
         <f aca="false">IF(OR(G51="",H51=""),"",G51-H51)</f>
         <v/>
       </c>
-      <c r="J51" s="46" t="str">
+      <c r="J51" s="55" t="str">
         <f aca="false">IF(OR(I51="",H51="",H51=0),"",I51/H51)</f>
         <v/>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47"/>
-      <c r="B52" s="22" t="str">
+      <c r="A52" s="56"/>
+      <c r="B52" s="41" t="str">
         <f aca="false">IF(A52="","",A52-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C52" s="22" t="str">
+      <c r="C52" s="41" t="str">
         <f aca="false">IF(A52="","",MIN(7,MAX(1,ROUNDUP(B52/7,0))))</f>
         <v/>
       </c>
-      <c r="D52" s="44" t="str">
+      <c r="D52" s="53" t="str">
         <f aca="false">IF(A52="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C52,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E52" s="48"/>
-      <c r="F52" s="48"/>
-      <c r="G52" s="19" t="str">
+      <c r="E52" s="57"/>
+      <c r="F52" s="57"/>
+      <c r="G52" s="38" t="str">
         <f aca="false">IF(E52="","",E52-IF(F52="",0,F52))</f>
         <v/>
       </c>
-      <c r="H52" s="19" t="str">
+      <c r="H52" s="38" t="str">
         <f aca="false">IF(A52="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C52,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I52" s="19" t="str">
+      <c r="I52" s="38" t="str">
         <f aca="false">IF(OR(G52="",H52=""),"",G52-H52)</f>
         <v/>
       </c>
-      <c r="J52" s="46" t="str">
+      <c r="J52" s="55" t="str">
         <f aca="false">IF(OR(I52="",H52="",H52=0),"",I52/H52)</f>
         <v/>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="47"/>
-      <c r="B53" s="22" t="str">
+      <c r="A53" s="56"/>
+      <c r="B53" s="41" t="str">
         <f aca="false">IF(A53="","",A53-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C53" s="22" t="str">
+      <c r="C53" s="41" t="str">
         <f aca="false">IF(A53="","",MIN(7,MAX(1,ROUNDUP(B53/7,0))))</f>
         <v/>
       </c>
-      <c r="D53" s="44" t="str">
+      <c r="D53" s="53" t="str">
         <f aca="false">IF(A53="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C53,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E53" s="48"/>
-      <c r="F53" s="48"/>
-      <c r="G53" s="19" t="str">
+      <c r="E53" s="57"/>
+      <c r="F53" s="57"/>
+      <c r="G53" s="38" t="str">
         <f aca="false">IF(E53="","",E53-IF(F53="",0,F53))</f>
         <v/>
       </c>
-      <c r="H53" s="19" t="str">
+      <c r="H53" s="38" t="str">
         <f aca="false">IF(A53="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C53,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I53" s="19" t="str">
+      <c r="I53" s="38" t="str">
         <f aca="false">IF(OR(G53="",H53=""),"",G53-H53)</f>
         <v/>
       </c>
-      <c r="J53" s="46" t="str">
+      <c r="J53" s="55" t="str">
         <f aca="false">IF(OR(I53="",H53="",H53=0),"",I53/H53)</f>
         <v/>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="47"/>
-      <c r="B54" s="22" t="str">
+      <c r="A54" s="56"/>
+      <c r="B54" s="41" t="str">
         <f aca="false">IF(A54="","",A54-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C54" s="22" t="str">
+      <c r="C54" s="41" t="str">
         <f aca="false">IF(A54="","",MIN(7,MAX(1,ROUNDUP(B54/7,0))))</f>
         <v/>
       </c>
-      <c r="D54" s="44" t="str">
+      <c r="D54" s="53" t="str">
         <f aca="false">IF(A54="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C54,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E54" s="48"/>
-      <c r="F54" s="48"/>
-      <c r="G54" s="19" t="str">
+      <c r="E54" s="57"/>
+      <c r="F54" s="57"/>
+      <c r="G54" s="38" t="str">
         <f aca="false">IF(E54="","",E54-IF(F54="",0,F54))</f>
         <v/>
       </c>
-      <c r="H54" s="19" t="str">
+      <c r="H54" s="38" t="str">
         <f aca="false">IF(A54="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C54,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I54" s="19" t="str">
+      <c r="I54" s="38" t="str">
         <f aca="false">IF(OR(G54="",H54=""),"",G54-H54)</f>
         <v/>
       </c>
-      <c r="J54" s="46" t="str">
+      <c r="J54" s="55" t="str">
         <f aca="false">IF(OR(I54="",H54="",H54=0),"",I54/H54)</f>
         <v/>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="47"/>
-      <c r="B55" s="22" t="str">
+      <c r="A55" s="56"/>
+      <c r="B55" s="41" t="str">
         <f aca="false">IF(A55="","",A55-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C55" s="22" t="str">
+      <c r="C55" s="41" t="str">
         <f aca="false">IF(A55="","",MIN(7,MAX(1,ROUNDUP(B55/7,0))))</f>
         <v/>
       </c>
-      <c r="D55" s="44" t="str">
+      <c r="D55" s="53" t="str">
         <f aca="false">IF(A55="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C55,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E55" s="48"/>
-      <c r="F55" s="48"/>
-      <c r="G55" s="19" t="str">
+      <c r="E55" s="57"/>
+      <c r="F55" s="57"/>
+      <c r="G55" s="38" t="str">
         <f aca="false">IF(E55="","",E55-IF(F55="",0,F55))</f>
         <v/>
       </c>
-      <c r="H55" s="19" t="str">
+      <c r="H55" s="38" t="str">
         <f aca="false">IF(A55="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C55,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I55" s="19" t="str">
+      <c r="I55" s="38" t="str">
         <f aca="false">IF(OR(G55="",H55=""),"",G55-H55)</f>
         <v/>
       </c>
-      <c r="J55" s="46" t="str">
+      <c r="J55" s="55" t="str">
         <f aca="false">IF(OR(I55="",H55="",H55=0),"",I55/H55)</f>
         <v/>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="47"/>
-      <c r="B56" s="22" t="str">
+      <c r="A56" s="56"/>
+      <c r="B56" s="41" t="str">
         <f aca="false">IF(A56="","",A56-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C56" s="22" t="str">
+      <c r="C56" s="41" t="str">
         <f aca="false">IF(A56="","",MIN(7,MAX(1,ROUNDUP(B56/7,0))))</f>
         <v/>
       </c>
-      <c r="D56" s="44" t="str">
+      <c r="D56" s="53" t="str">
         <f aca="false">IF(A56="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C56,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E56" s="48"/>
-      <c r="F56" s="48"/>
-      <c r="G56" s="19" t="str">
+      <c r="E56" s="57"/>
+      <c r="F56" s="57"/>
+      <c r="G56" s="38" t="str">
         <f aca="false">IF(E56="","",E56-IF(F56="",0,F56))</f>
         <v/>
       </c>
-      <c r="H56" s="19" t="str">
+      <c r="H56" s="38" t="str">
         <f aca="false">IF(A56="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C56,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I56" s="19" t="str">
+      <c r="I56" s="38" t="str">
         <f aca="false">IF(OR(G56="",H56=""),"",G56-H56)</f>
         <v/>
       </c>
-      <c r="J56" s="46" t="str">
+      <c r="J56" s="55" t="str">
         <f aca="false">IF(OR(I56="",H56="",H56=0),"",I56/H56)</f>
         <v/>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="47"/>
-      <c r="B57" s="22" t="str">
+      <c r="A57" s="56"/>
+      <c r="B57" s="41" t="str">
         <f aca="false">IF(A57="","",A57-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C57" s="22" t="str">
+      <c r="C57" s="41" t="str">
         <f aca="false">IF(A57="","",MIN(7,MAX(1,ROUNDUP(B57/7,0))))</f>
         <v/>
       </c>
-      <c r="D57" s="44" t="str">
+      <c r="D57" s="53" t="str">
         <f aca="false">IF(A57="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C57,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E57" s="48"/>
-      <c r="F57" s="48"/>
-      <c r="G57" s="19" t="str">
+      <c r="E57" s="57"/>
+      <c r="F57" s="57"/>
+      <c r="G57" s="38" t="str">
         <f aca="false">IF(E57="","",E57-IF(F57="",0,F57))</f>
         <v/>
       </c>
-      <c r="H57" s="19" t="str">
+      <c r="H57" s="38" t="str">
         <f aca="false">IF(A57="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C57,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I57" s="19" t="str">
+      <c r="I57" s="38" t="str">
         <f aca="false">IF(OR(G57="",H57=""),"",G57-H57)</f>
         <v/>
       </c>
-      <c r="J57" s="46" t="str">
+      <c r="J57" s="55" t="str">
         <f aca="false">IF(OR(I57="",H57="",H57=0),"",I57/H57)</f>
         <v/>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="47"/>
-      <c r="B58" s="22" t="str">
+      <c r="A58" s="56"/>
+      <c r="B58" s="41" t="str">
         <f aca="false">IF(A58="","",A58-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C58" s="22" t="str">
+      <c r="C58" s="41" t="str">
         <f aca="false">IF(A58="","",MIN(7,MAX(1,ROUNDUP(B58/7,0))))</f>
         <v/>
       </c>
-      <c r="D58" s="44" t="str">
+      <c r="D58" s="53" t="str">
         <f aca="false">IF(A58="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C58,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E58" s="48"/>
-      <c r="F58" s="48"/>
-      <c r="G58" s="19" t="str">
+      <c r="E58" s="57"/>
+      <c r="F58" s="57"/>
+      <c r="G58" s="38" t="str">
         <f aca="false">IF(E58="","",E58-IF(F58="",0,F58))</f>
         <v/>
       </c>
-      <c r="H58" s="19" t="str">
+      <c r="H58" s="38" t="str">
         <f aca="false">IF(A58="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C58,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I58" s="19" t="str">
+      <c r="I58" s="38" t="str">
         <f aca="false">IF(OR(G58="",H58=""),"",G58-H58)</f>
         <v/>
       </c>
-      <c r="J58" s="46" t="str">
+      <c r="J58" s="55" t="str">
         <f aca="false">IF(OR(I58="",H58="",H58=0),"",I58/H58)</f>
         <v/>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="47"/>
-      <c r="B59" s="22" t="str">
+      <c r="A59" s="56"/>
+      <c r="B59" s="41" t="str">
         <f aca="false">IF(A59="","",A59-FechaInicioLote+1)</f>
         <v/>
       </c>
-      <c r="C59" s="22" t="str">
+      <c r="C59" s="41" t="str">
         <f aca="false">IF(A59="","",MIN(7,MAX(1,ROUNDUP(B59/7,0))))</f>
         <v/>
       </c>
-      <c r="D59" s="44" t="str">
+      <c r="D59" s="53" t="str">
         <f aca="false">IF(A59="","",INDEX('Tabla Tecnica Base'!$B$4:$B$10,MATCH(C59,'Tabla Tecnica Base'!$A$4:$A$10,0)))</f>
         <v/>
       </c>
-      <c r="E59" s="48"/>
-      <c r="F59" s="48"/>
-      <c r="G59" s="19" t="str">
+      <c r="E59" s="57"/>
+      <c r="F59" s="57"/>
+      <c r="G59" s="38" t="str">
         <f aca="false">IF(E59="","",E59-IF(F59="",0,F59))</f>
         <v/>
       </c>
-      <c r="H59" s="19" t="str">
+      <c r="H59" s="38" t="str">
         <f aca="false">IF(A59="","",INDEX('Tabla Tecnica Base'!$E$4:$E$10,MATCH(C59,'Tabla Tecnica Base'!$A$4:$A$10,0))/1000*CantidadPollos)</f>
         <v/>
       </c>
-      <c r="I59" s="19" t="str">
+      <c r="I59" s="38" t="str">
         <f aca="false">IF(OR(G59="",H59=""),"",G59-H59)</f>
         <v/>
       </c>
-      <c r="J59" s="46" t="str">
+      <c r="J59" s="55" t="str">
         <f aca="false">IF(OR(I59="",H59="",H59=0),"",I59/H59)</f>
         <v/>
       </c>
@@ -4125,21 +4247,21 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
+      <c r="A1" s="34" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4151,210 +4273,176 @@
       <c r="I2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>73</v>
-      </c>
-      <c r="H3" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>75</v>
+      <c r="A3" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="C4" s="37" t="s">
-        <v>77</v>
-      </c>
-      <c r="D4" s="19" t="n">
+      <c r="A4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="38" t="n">
         <f aca="false">E4/CantidadPollos</f>
-        <v>0.126</v>
-      </c>
-      <c r="E4" s="20" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="E4" s="39" t="n">
         <f aca="false">SUMIF('Tabla Semanal'!$B$4:$B$10,A4,'Tabla Semanal'!$H$4:$H$10)</f>
-        <v>12.6</v>
-      </c>
-      <c r="F4" s="19" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="F4" s="38" t="n">
         <f aca="false">E4/PesoBulto</f>
-        <v>0.315</v>
-      </c>
-      <c r="G4" s="21" t="n">
+        <v>2.205</v>
+      </c>
+      <c r="G4" s="40" t="n">
         <f aca="false">ROUNDUP(F4,0)</f>
-        <v>1</v>
-      </c>
-      <c r="H4" s="50" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="I4" s="51" t="n">
+      <c r="I4" s="59" t="n">
         <f aca="false">G4*H4</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="52" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="39" t="s">
-        <v>78</v>
-      </c>
-      <c r="C5" s="39" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="19" t="n">
+      <c r="A5" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="38" t="n">
         <f aca="false">E5/CantidadPollos</f>
-        <v>0.756</v>
-      </c>
-      <c r="E5" s="20" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="E5" s="39" t="n">
         <f aca="false">SUMIF('Tabla Semanal'!$B$4:$B$10,A5,'Tabla Semanal'!$H$4:$H$10)</f>
-        <v>75.6</v>
-      </c>
-      <c r="F5" s="19" t="n">
+        <v>147</v>
+      </c>
+      <c r="F5" s="38" t="n">
         <f aca="false">E5/PesoBulto</f>
-        <v>1.89</v>
-      </c>
-      <c r="G5" s="21" t="n">
+        <v>3.675</v>
+      </c>
+      <c r="G5" s="40" t="n">
         <f aca="false">ROUNDUP(F5,0)</f>
-        <v>2</v>
-      </c>
-      <c r="H5" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="51" t="n">
+      <c r="I5" s="59" t="n">
         <f aca="false">G5*H5</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="53" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="40" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="40" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="19" t="n">
+      <c r="A6" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="38" t="n">
         <f aca="false">E6/CantidadPollos</f>
-        <v>1.47</v>
-      </c>
-      <c r="E6" s="20" t="n">
+        <v>2.114</v>
+      </c>
+      <c r="E6" s="39" t="n">
         <f aca="false">SUMIF('Tabla Semanal'!$B$4:$B$10,A6,'Tabla Semanal'!$H$4:$H$10)</f>
-        <v>147</v>
-      </c>
-      <c r="F6" s="19" t="n">
+        <v>211.4</v>
+      </c>
+      <c r="F6" s="38" t="n">
         <f aca="false">E6/PesoBulto</f>
-        <v>3.675</v>
-      </c>
-      <c r="G6" s="21" t="n">
+        <v>5.285</v>
+      </c>
+      <c r="G6" s="40" t="n">
         <f aca="false">ROUNDUP(F6,0)</f>
-        <v>4</v>
-      </c>
-      <c r="H6" s="50" t="n">
+        <v>6</v>
+      </c>
+      <c r="H6" s="58" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="51" t="n">
+      <c r="I6" s="59" t="n">
         <f aca="false">G6*H6</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="54" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" s="41" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7" s="41" t="s">
-        <v>83</v>
-      </c>
-      <c r="D7" s="19" t="n">
-        <f aca="false">E7/CantidadPollos</f>
-        <v>2.114</v>
-      </c>
-      <c r="E7" s="20" t="n">
-        <f aca="false">SUMIF('Tabla Semanal'!$B$4:$B$10,A7,'Tabla Semanal'!$H$4:$H$10)</f>
-        <v>211.4</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <f aca="false">E7/PesoBulto</f>
-        <v>5.285</v>
-      </c>
-      <c r="G7" s="21" t="n">
-        <f aca="false">ROUNDUP(F7,0)</f>
-        <v>6</v>
-      </c>
-      <c r="H7" s="50" t="n">
+      <c r="A7" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="26" t="n">
+        <f aca="false">SUM(D4:D6)</f>
+        <v>4.466</v>
+      </c>
+      <c r="E7" s="26" t="n">
+        <f aca="false">SUM(E4:E6)</f>
+        <v>446.6</v>
+      </c>
+      <c r="F7" s="49" t="n">
+        <f aca="false">SUM(F4:F6)</f>
+        <v>11.165</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <f aca="false">SUM(G4:G6)</f>
+        <v>13</v>
+      </c>
+      <c r="H7" s="60"/>
+      <c r="I7" s="61" t="n">
+        <f aca="false">SUM(I4:I6)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="51" t="n">
-        <f aca="false">G7*H7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="55" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="34" t="n">
-        <f aca="false">SUM(D4:D7)</f>
-        <v>4.466</v>
-      </c>
-      <c r="E8" s="34" t="n">
-        <f aca="false">SUM(E4:E7)</f>
-        <v>446.6</v>
-      </c>
-      <c r="F8" s="35" t="n">
-        <f aca="false">SUM(F4:F7)</f>
-        <v>11.165</v>
-      </c>
-      <c r="G8" s="36" t="n">
-        <f aca="false">SUM(G4:G7)</f>
-        <v>13</v>
-      </c>
-      <c r="H8" s="56"/>
-      <c r="I8" s="57" t="n">
-        <f aca="false">SUM(I4:I7)</f>
-        <v>0</v>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="13"/>
+      <c r="A10" s="33" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="33"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="33"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4387,69 +4475,69 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="58" t="s">
-        <v>87</v>
-      </c>
-      <c r="B3" s="58"/>
-    </row>
-    <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="59" t="s">
+      <c r="A3" s="62" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="59"/>
+      <c r="B3" s="62"/>
+    </row>
+    <row r="4" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="63" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="63"/>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="58" t="s">
-        <v>89</v>
-      </c>
-      <c r="B5" s="58"/>
+      <c r="A5" s="62" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="62"/>
     </row>
     <row r="6" customFormat="false" ht="75.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="59" t="s">
-        <v>90</v>
-      </c>
-      <c r="B6" s="59"/>
+      <c r="A6" s="63" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="63"/>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="58" t="s">
-        <v>91</v>
-      </c>
-      <c r="B7" s="58"/>
+      <c r="A7" s="62" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="62"/>
     </row>
     <row r="8" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="59" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" s="59"/>
+      <c r="A8" s="63" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="63"/>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="58" t="s">
-        <v>93</v>
-      </c>
-      <c r="B9" s="58"/>
+      <c r="A9" s="62" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="62"/>
     </row>
     <row r="10" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="59" t="s">
-        <v>94</v>
-      </c>
-      <c r="B10" s="59"/>
+      <c r="A10" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" s="63"/>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="B11" s="58"/>
+      <c r="A11" s="62" t="s">
+        <v>96</v>
+      </c>
+      <c r="B11" s="62"/>
     </row>
     <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="59" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" s="59"/>
+      <c r="A12" s="63" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="63"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>